<commit_message>
revert row-20 table, redo edit confined to rows 17-19 (user feedback)
Itemize in Analysis Purpose field, not a new inserted table; rows 20+ untouched.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
+++ b/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
@@ -101,7 +101,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="42">
+  <borders count="37">
     <border>
       <left/>
       <right/>
@@ -358,41 +358,6 @@
       <left/>
       <right style="medium"/>
       <top/>
-      <bottom style="medium"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
       <bottom style="medium"/>
       <diagonal/>
     </border>
@@ -407,7 +372,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -622,36 +587,6 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
@@ -994,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H53"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38.44" customWidth="1" style="46" min="1" max="1"/>
@@ -1223,7 +1158,8 @@
       <c r="B17" s="76" t="inlineStr">
         <is>
           <t>The analysis type (input only ONE type of analysis), such as 
-RNAseq,  Single-Cell-Analysis, spatial Transcriptomics, whole-genome-sequence, proteomics, mapping based or assembly-based shotgun metagenomics</t>
+RNAseq,  Single-Cell-Analysis, spatial Transcriptomics, whole-genome-sequence, proteomics, mapping based or assembly-based shotgun metagenomics
+⚠ If this submission includes two different analysis types or two distinct parts (e.g. RNAseq AND WGS, or two separate studies), please fill out and submit TWO separate copies of this form, one per analysis type / part.</t>
         </is>
       </c>
       <c r="C17" s="64" t="n"/>
@@ -1233,17 +1169,25 @@
       <c r="G17" s="64" t="n"/>
       <c r="H17" s="65" t="n"/>
     </row>
-    <row r="18" ht="33" customHeight="1" s="47">
+    <row r="18" ht="165" customHeight="1" s="47">
       <c r="A18" s="77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Analysis Purpose 
-And Setting </t>
+          <t>Analysis Purpose
+And Setting
+(list EACH
+requirement as its
+own numbered line)</t>
         </is>
       </c>
       <c r="B18" s="78" t="inlineStr">
         <is>
-          <t xml:space="preserve">The Specific analysis instruciton (input ALL necessary requirements), such as 
-Such as analysis purpose, how to filter, groups to be compared with, which is the control group (if applicable),        </t>
+          <t xml:space="preserve">List EVERY requirement as its own numbered line below — e.g. analysis purpose, filtering/QC thresholds, groups to be compared, which is the control group (if applicable), statistical tests/significance thresholds, specific outputs needed. Do not combine multiple requirements into one line; add or delete numbered lines as needed.
+1. 
+2. 
+3. 
+4. 
+5. 
+6. </t>
         </is>
       </c>
       <c r="C18" s="64" t="n"/>
@@ -1259,16 +1203,19 @@
           <t>Analysis requirements:
 Regular work for your selected category
 have no extra fee.
-Custom requirements has additional fee
-($120/h). Our specialist will tell you
-which item is Custom.
-⚠ IMPORTANT: List EVERY requirement as
-its own row in the table below. This form
-is the SOLE basis for analysis scope and
-pricing — requirements communicated only
-verbally or by email, and not entered here,
-will NOT be included in the analysis or the
-quote unless this form is updated and
+Custom requirements has Additional fee
+($120/h).
+Our specialist will tell you which one is
+Custom item.
+⚠ IMPORTANT: This form — Sample Note +
+Analysis Type + Analysis Purpose and
+Setting above — is the SOLE basis for
+analysis scope and pricing. Requirements
+communicated only verbally or by email,
+and not written in the Analysis Purpose
+and Setting field above, will NOT be
+included in the analysis or the quote
+unless this form is updated and
 re-submitted.</t>
         </is>
       </c>
@@ -1290,555 +1237,400 @@
       <c r="G19" s="64" t="n"/>
       <c r="H19" s="65" t="n"/>
     </row>
-    <row r="20" ht="30" customHeight="1" s="47">
-      <c r="A20" s="81" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B20" s="82" t="inlineStr">
-        <is>
-          <t>Requirement Description — list ONE specific requirement per row</t>
-        </is>
-      </c>
-      <c r="C20" s="68" t="n"/>
-      <c r="D20" s="68" t="n"/>
-      <c r="E20" s="68" t="n"/>
-      <c r="F20" s="83" t="n"/>
-      <c r="G20" s="82" t="inlineStr">
-        <is>
-          <t>Regular / Custom
-(specialist to complete)</t>
-        </is>
-      </c>
-      <c r="H20" s="84" t="inlineStr">
-        <is>
-          <t>Notes / Est. Hours
-(if Custom, $120/h)</t>
-        </is>
-      </c>
+    <row r="20" ht="15" customHeight="1" s="47">
+      <c r="A20" s="55" t="inlineStr">
+        <is>
+          <t>Example 1</t>
+        </is>
+      </c>
+      <c r="B20" s="81" t="n"/>
+      <c r="C20" s="81" t="n"/>
+      <c r="D20" s="81" t="n"/>
+      <c r="E20" s="81" t="n"/>
+      <c r="F20" s="81" t="n"/>
+      <c r="G20" s="81" t="n"/>
+      <c r="H20" s="82" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="47">
-      <c r="A21" s="85" t="n">
-        <v>1</v>
-      </c>
-      <c r="B21" s="93" t="n"/>
-      <c r="C21" s="57" t="n"/>
-      <c r="D21" s="57" t="n"/>
-      <c r="E21" s="57" t="n"/>
-      <c r="F21" s="87" t="n"/>
-      <c r="G21" s="93" t="n"/>
-      <c r="H21" s="94" t="n"/>
+      <c r="A21" s="55" t="inlineStr">
+        <is>
+          <t>Example 2</t>
+        </is>
+      </c>
+      <c r="B21" s="81" t="n"/>
+      <c r="C21" s="81" t="n"/>
+      <c r="D21" s="81" t="n"/>
+      <c r="E21" s="81" t="n"/>
+      <c r="F21" s="81" t="n"/>
+      <c r="G21" s="81" t="n"/>
+      <c r="H21" s="82" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="47">
-      <c r="A22" s="85" t="n">
-        <v>2</v>
-      </c>
-      <c r="B22" s="93" t="n"/>
-      <c r="C22" s="57" t="n"/>
-      <c r="D22" s="57" t="n"/>
-      <c r="E22" s="57" t="n"/>
-      <c r="F22" s="87" t="n"/>
-      <c r="G22" s="93" t="n"/>
-      <c r="H22" s="94" t="n"/>
+      <c r="A22" s="55" t="inlineStr">
+        <is>
+          <t>Example 3</t>
+        </is>
+      </c>
+      <c r="B22" s="81" t="n"/>
+      <c r="C22" s="81" t="n"/>
+      <c r="D22" s="81" t="n"/>
+      <c r="E22" s="81" t="n"/>
+      <c r="F22" s="81" t="n"/>
+      <c r="G22" s="81" t="n"/>
+      <c r="H22" s="82" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="47">
-      <c r="A23" s="85" t="n">
-        <v>3</v>
-      </c>
-      <c r="B23" s="93" t="n"/>
-      <c r="C23" s="57" t="n"/>
-      <c r="D23" s="57" t="n"/>
-      <c r="E23" s="57" t="n"/>
-      <c r="F23" s="87" t="n"/>
-      <c r="G23" s="93" t="n"/>
-      <c r="H23" s="94" t="n"/>
+      <c r="A23" s="55" t="inlineStr">
+        <is>
+          <t>Example 4</t>
+        </is>
+      </c>
+      <c r="B23" s="81" t="n"/>
+      <c r="C23" s="81" t="n"/>
+      <c r="D23" s="81" t="n"/>
+      <c r="E23" s="81" t="n"/>
+      <c r="F23" s="81" t="n"/>
+      <c r="G23" s="81" t="n"/>
+      <c r="H23" s="82" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="47">
-      <c r="A24" s="85" t="n">
-        <v>4</v>
-      </c>
-      <c r="B24" s="93" t="n"/>
-      <c r="C24" s="57" t="n"/>
-      <c r="D24" s="57" t="n"/>
-      <c r="E24" s="57" t="n"/>
-      <c r="F24" s="87" t="n"/>
-      <c r="G24" s="93" t="n"/>
-      <c r="H24" s="94" t="n"/>
+      <c r="A24" s="55" t="inlineStr">
+        <is>
+          <t>Example 5</t>
+        </is>
+      </c>
+      <c r="B24" s="81" t="n"/>
+      <c r="C24" s="81" t="n"/>
+      <c r="D24" s="81" t="n"/>
+      <c r="E24" s="81" t="n"/>
+      <c r="F24" s="81" t="n"/>
+      <c r="G24" s="81" t="n"/>
+      <c r="H24" s="82" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="47">
-      <c r="A25" s="85" t="n">
-        <v>5</v>
-      </c>
-      <c r="B25" s="93" t="n"/>
-      <c r="C25" s="57" t="n"/>
-      <c r="D25" s="57" t="n"/>
-      <c r="E25" s="57" t="n"/>
-      <c r="F25" s="87" t="n"/>
-      <c r="G25" s="93" t="n"/>
-      <c r="H25" s="94" t="n"/>
+      <c r="A25" s="55" t="inlineStr">
+        <is>
+          <t>Example 6</t>
+        </is>
+      </c>
+      <c r="B25" s="81" t="n"/>
+      <c r="C25" s="81" t="n"/>
+      <c r="D25" s="81" t="n"/>
+      <c r="E25" s="81" t="n"/>
+      <c r="F25" s="81" t="n"/>
+      <c r="G25" s="81" t="n"/>
+      <c r="H25" s="82" t="n"/>
     </row>
     <row r="26" ht="15" customHeight="1" s="47">
-      <c r="A26" s="85" t="n">
-        <v>6</v>
-      </c>
-      <c r="B26" s="93" t="n"/>
-      <c r="C26" s="57" t="n"/>
-      <c r="D26" s="57" t="n"/>
-      <c r="E26" s="57" t="n"/>
-      <c r="F26" s="87" t="n"/>
-      <c r="G26" s="93" t="n"/>
-      <c r="H26" s="94" t="n"/>
+      <c r="A26" s="55" t="inlineStr">
+        <is>
+          <t>Example 7</t>
+        </is>
+      </c>
+      <c r="B26" s="81" t="n"/>
+      <c r="C26" s="81" t="n"/>
+      <c r="D26" s="81" t="n"/>
+      <c r="E26" s="81" t="n"/>
+      <c r="F26" s="81" t="n"/>
+      <c r="G26" s="81" t="n"/>
+      <c r="H26" s="82" t="n"/>
     </row>
     <row r="27" ht="15" customHeight="1" s="47">
-      <c r="A27" s="85" t="n">
-        <v>7</v>
-      </c>
-      <c r="B27" s="93" t="n"/>
-      <c r="C27" s="57" t="n"/>
-      <c r="D27" s="57" t="n"/>
-      <c r="E27" s="57" t="n"/>
-      <c r="F27" s="87" t="n"/>
-      <c r="G27" s="93" t="n"/>
-      <c r="H27" s="94" t="n"/>
+      <c r="A27" s="55" t="inlineStr">
+        <is>
+          <t>Example 8</t>
+        </is>
+      </c>
+      <c r="B27" s="81" t="n"/>
+      <c r="C27" s="81" t="n"/>
+      <c r="D27" s="81" t="n"/>
+      <c r="E27" s="81" t="n"/>
+      <c r="F27" s="81" t="n"/>
+      <c r="G27" s="81" t="n"/>
+      <c r="H27" s="82" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="47">
-      <c r="A28" s="85" t="n">
-        <v>8</v>
-      </c>
-      <c r="B28" s="93" t="n"/>
-      <c r="C28" s="57" t="n"/>
-      <c r="D28" s="57" t="n"/>
-      <c r="E28" s="57" t="n"/>
-      <c r="F28" s="87" t="n"/>
-      <c r="G28" s="93" t="n"/>
-      <c r="H28" s="94" t="n"/>
+      <c r="A28" s="55" t="inlineStr">
+        <is>
+          <t>Example 9</t>
+        </is>
+      </c>
+      <c r="B28" s="81" t="n"/>
+      <c r="C28" s="81" t="n"/>
+      <c r="D28" s="81" t="n"/>
+      <c r="E28" s="81" t="n"/>
+      <c r="F28" s="81" t="n"/>
+      <c r="G28" s="81" t="n"/>
+      <c r="H28" s="82" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="47">
-      <c r="A29" s="85" t="n">
-        <v>9</v>
-      </c>
-      <c r="B29" s="93" t="n"/>
-      <c r="C29" s="57" t="n"/>
-      <c r="D29" s="57" t="n"/>
-      <c r="E29" s="57" t="n"/>
-      <c r="F29" s="87" t="n"/>
-      <c r="G29" s="93" t="n"/>
-      <c r="H29" s="94" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="47">
-      <c r="A30" s="89" t="n">
-        <v>10</v>
-      </c>
-      <c r="B30" s="95" t="n"/>
-      <c r="C30" s="61" t="n"/>
-      <c r="D30" s="61" t="n"/>
-      <c r="E30" s="61" t="n"/>
-      <c r="F30" s="91" t="n"/>
-      <c r="G30" s="95" t="n"/>
-      <c r="H30" s="96" t="n"/>
-    </row>
+      <c r="A29" s="59" t="inlineStr">
+        <is>
+          <t>Example 10</t>
+        </is>
+      </c>
+      <c r="B29" s="83" t="n"/>
+      <c r="C29" s="83" t="n"/>
+      <c r="D29" s="83" t="n"/>
+      <c r="E29" s="83" t="n"/>
+      <c r="F29" s="83" t="n"/>
+      <c r="G29" s="83" t="n"/>
+      <c r="H29" s="84" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="47"/>
     <row r="31" ht="15" customHeight="1" s="47">
-      <c r="A31" s="55" t="inlineStr">
-        <is>
-          <t>Example 1</t>
-        </is>
-      </c>
+      <c r="A31" s="63" t="inlineStr">
+        <is>
+          <t>Nucleic Acids Additional Information</t>
+        </is>
+      </c>
+      <c r="B31" s="64" t="n"/>
+      <c r="C31" s="64" t="n"/>
+      <c r="D31" s="64" t="n"/>
+      <c r="E31" s="64" t="n"/>
+      <c r="F31" s="64" t="n"/>
+      <c r="G31" s="64" t="n"/>
+      <c r="H31" s="65" t="n"/>
     </row>
     <row r="32" ht="14.25" customHeight="1" s="47">
-      <c r="A32" s="55" t="inlineStr">
-        <is>
-          <t>Example 2</t>
-        </is>
-      </c>
-      <c r="B32" s="93" t="n"/>
-      <c r="C32" s="93" t="n"/>
-      <c r="D32" s="93" t="n"/>
-      <c r="E32" s="93" t="n"/>
-      <c r="F32" s="93" t="n"/>
-      <c r="G32" s="93" t="n"/>
-      <c r="H32" s="94" t="n"/>
+      <c r="A32" s="66" t="inlineStr">
+        <is>
+          <t>Sample Name</t>
+        </is>
+      </c>
+      <c r="B32" s="85" t="inlineStr">
+        <is>
+          <t>Nucleic Acid Type</t>
+        </is>
+      </c>
+      <c r="C32" s="85" t="inlineStr">
+        <is>
+          <t>Storage Reagent</t>
+        </is>
+      </c>
+      <c r="D32" s="85" t="inlineStr">
+        <is>
+          <t>Concentration (ng/µL)</t>
+        </is>
+      </c>
+      <c r="E32" s="85" t="inlineStr">
+        <is>
+          <t>Volume (µL)</t>
+        </is>
+      </c>
+      <c r="F32" s="85" t="inlineStr">
+        <is>
+          <t>Size (bp, if applicable)</t>
+        </is>
+      </c>
+      <c r="G32" s="85" t="inlineStr">
+        <is>
+          <t>i7 Index (if any)</t>
+        </is>
+      </c>
+      <c r="H32" s="86" t="inlineStr">
+        <is>
+          <t>i5 Index (NovaSeq 1.0/Forward)</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="47">
       <c r="A33" s="55" t="inlineStr">
         <is>
-          <t>Example 3</t>
-        </is>
-      </c>
-      <c r="B33" s="93" t="n"/>
-      <c r="C33" s="93" t="n"/>
-      <c r="D33" s="93" t="n"/>
-      <c r="E33" s="93" t="n"/>
-      <c r="F33" s="93" t="n"/>
-      <c r="G33" s="93" t="n"/>
-      <c r="H33" s="94" t="n"/>
+          <t>Example 1</t>
+        </is>
+      </c>
+      <c r="B33" s="81" t="n"/>
+      <c r="C33" s="81" t="n"/>
+      <c r="D33" s="81" t="n"/>
+      <c r="E33" s="81" t="n"/>
+      <c r="F33" s="81" t="n"/>
+      <c r="G33" s="81" t="n"/>
+      <c r="H33" s="82" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="47">
       <c r="A34" s="55" t="inlineStr">
         <is>
-          <t>Example 4</t>
-        </is>
-      </c>
-      <c r="B34" s="93" t="n"/>
-      <c r="C34" s="93" t="n"/>
-      <c r="D34" s="93" t="n"/>
-      <c r="E34" s="93" t="n"/>
-      <c r="F34" s="93" t="n"/>
-      <c r="G34" s="93" t="n"/>
-      <c r="H34" s="94" t="n"/>
+          <t>Example 2</t>
+        </is>
+      </c>
+      <c r="B34" s="81" t="n"/>
+      <c r="C34" s="81" t="n"/>
+      <c r="D34" s="81" t="n"/>
+      <c r="E34" s="81" t="n"/>
+      <c r="F34" s="81" t="n"/>
+      <c r="G34" s="81" t="n"/>
+      <c r="H34" s="82" t="n"/>
     </row>
     <row r="35" ht="14.25" customHeight="1" s="47">
       <c r="A35" s="55" t="inlineStr">
         <is>
-          <t>Example 5</t>
-        </is>
-      </c>
-      <c r="B35" s="93" t="n"/>
-      <c r="C35" s="93" t="n"/>
-      <c r="D35" s="93" t="n"/>
-      <c r="E35" s="93" t="n"/>
-      <c r="F35" s="93" t="n"/>
-      <c r="G35" s="93" t="n"/>
-      <c r="H35" s="94" t="n"/>
+          <t>Example 3</t>
+        </is>
+      </c>
+      <c r="B35" s="81" t="n"/>
+      <c r="C35" s="81" t="n"/>
+      <c r="D35" s="81" t="n"/>
+      <c r="E35" s="81" t="n"/>
+      <c r="F35" s="81" t="n"/>
+      <c r="G35" s="81" t="n"/>
+      <c r="H35" s="82" t="n"/>
     </row>
     <row r="36" ht="14.25" customHeight="1" s="47">
       <c r="A36" s="55" t="inlineStr">
         <is>
-          <t>Example 6</t>
-        </is>
-      </c>
-      <c r="B36" s="93" t="n"/>
-      <c r="C36" s="93" t="n"/>
-      <c r="D36" s="93" t="n"/>
-      <c r="E36" s="93" t="n"/>
-      <c r="F36" s="93" t="n"/>
-      <c r="G36" s="93" t="n"/>
-      <c r="H36" s="94" t="n"/>
+          <t>Example 4</t>
+        </is>
+      </c>
+      <c r="B36" s="81" t="n"/>
+      <c r="C36" s="81" t="n"/>
+      <c r="D36" s="81" t="n"/>
+      <c r="E36" s="81" t="n"/>
+      <c r="F36" s="81" t="n"/>
+      <c r="G36" s="81" t="n"/>
+      <c r="H36" s="82" t="n"/>
     </row>
     <row r="37" ht="14.25" customHeight="1" s="47">
       <c r="A37" s="55" t="inlineStr">
         <is>
-          <t>Example 7</t>
-        </is>
-      </c>
-      <c r="B37" s="93" t="n"/>
-      <c r="C37" s="93" t="n"/>
-      <c r="D37" s="93" t="n"/>
-      <c r="E37" s="93" t="n"/>
-      <c r="F37" s="93" t="n"/>
-      <c r="G37" s="93" t="n"/>
-      <c r="H37" s="94" t="n"/>
+          <t>Example 5</t>
+        </is>
+      </c>
+      <c r="B37" s="81" t="n"/>
+      <c r="C37" s="81" t="n"/>
+      <c r="D37" s="81" t="n"/>
+      <c r="E37" s="81" t="n"/>
+      <c r="F37" s="81" t="n"/>
+      <c r="G37" s="81" t="n"/>
+      <c r="H37" s="82" t="n"/>
     </row>
     <row r="38" ht="14.25" customHeight="1" s="47">
       <c r="A38" s="55" t="inlineStr">
         <is>
-          <t>Example 8</t>
-        </is>
-      </c>
-      <c r="B38" s="93" t="n"/>
-      <c r="C38" s="93" t="n"/>
-      <c r="D38" s="93" t="n"/>
-      <c r="E38" s="93" t="n"/>
-      <c r="F38" s="93" t="n"/>
-      <c r="G38" s="93" t="n"/>
-      <c r="H38" s="94" t="n"/>
+          <t>Example 6</t>
+        </is>
+      </c>
+      <c r="B38" s="81" t="n"/>
+      <c r="C38" s="81" t="n"/>
+      <c r="D38" s="81" t="n"/>
+      <c r="E38" s="81" t="n"/>
+      <c r="F38" s="81" t="n"/>
+      <c r="G38" s="81" t="n"/>
+      <c r="H38" s="82" t="n"/>
     </row>
     <row r="39" ht="14.25" customHeight="1" s="47">
       <c r="A39" s="55" t="inlineStr">
         <is>
+          <t>Example 7</t>
+        </is>
+      </c>
+      <c r="B39" s="81" t="n"/>
+      <c r="C39" s="81" t="n"/>
+      <c r="D39" s="81" t="n"/>
+      <c r="E39" s="81" t="n"/>
+      <c r="F39" s="81" t="n"/>
+      <c r="G39" s="81" t="n"/>
+      <c r="H39" s="82" t="n"/>
+    </row>
+    <row r="40" ht="14.25" customHeight="1" s="47">
+      <c r="A40" s="55" t="inlineStr">
+        <is>
+          <t>Example 8</t>
+        </is>
+      </c>
+      <c r="B40" s="81" t="n"/>
+      <c r="C40" s="81" t="n"/>
+      <c r="D40" s="81" t="n"/>
+      <c r="E40" s="81" t="n"/>
+      <c r="F40" s="81" t="n"/>
+      <c r="G40" s="81" t="n"/>
+      <c r="H40" s="82" t="n"/>
+    </row>
+    <row r="41" ht="14.25" customHeight="1" s="47">
+      <c r="A41" s="55" t="inlineStr">
+        <is>
           <t>Example 9</t>
         </is>
       </c>
-      <c r="B39" s="93" t="n"/>
-      <c r="C39" s="93" t="n"/>
-      <c r="D39" s="93" t="n"/>
-      <c r="E39" s="93" t="n"/>
-      <c r="F39" s="93" t="n"/>
-      <c r="G39" s="93" t="n"/>
-      <c r="H39" s="94" t="n"/>
-    </row>
-    <row r="40" ht="14.25" customHeight="1" s="47">
-      <c r="A40" s="59" t="inlineStr">
+      <c r="B41" s="81" t="n"/>
+      <c r="C41" s="81" t="n"/>
+      <c r="D41" s="81" t="n"/>
+      <c r="E41" s="81" t="n"/>
+      <c r="F41" s="81" t="n"/>
+      <c r="G41" s="81" t="n"/>
+      <c r="H41" s="82" t="n"/>
+    </row>
+    <row r="42" ht="15" customHeight="1" s="47">
+      <c r="A42" s="59" t="inlineStr">
         <is>
           <t>Example 10</t>
         </is>
       </c>
-      <c r="B40" s="95" t="n"/>
-      <c r="C40" s="95" t="n"/>
-      <c r="D40" s="95" t="n"/>
-      <c r="E40" s="95" t="n"/>
-      <c r="F40" s="95" t="n"/>
-      <c r="G40" s="95" t="n"/>
-      <c r="H40" s="96" t="n"/>
-    </row>
-    <row r="41" ht="14.25" customHeight="1" s="47"/>
-    <row r="42" ht="15" customHeight="1" s="47">
-      <c r="A42" s="63" t="inlineStr">
-        <is>
-          <t>Nucleic Acids Additional Information</t>
-        </is>
-      </c>
-      <c r="B42" s="64" t="n"/>
-      <c r="C42" s="64" t="n"/>
-      <c r="D42" s="64" t="n"/>
-      <c r="E42" s="64" t="n"/>
-      <c r="F42" s="64" t="n"/>
-      <c r="G42" s="64" t="n"/>
-      <c r="H42" s="65" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="66" t="inlineStr">
-        <is>
-          <t>Sample Name</t>
-        </is>
-      </c>
-      <c r="B43" s="97" t="inlineStr">
-        <is>
-          <t>Nucleic Acid Type</t>
-        </is>
-      </c>
-      <c r="C43" s="97" t="inlineStr">
-        <is>
-          <t>Storage Reagent</t>
-        </is>
-      </c>
-      <c r="D43" s="97" t="inlineStr">
-        <is>
-          <t>Concentration (ng/µL)</t>
-        </is>
-      </c>
-      <c r="E43" s="97" t="inlineStr">
-        <is>
-          <t>Volume (µL)</t>
-        </is>
-      </c>
-      <c r="F43" s="97" t="inlineStr">
-        <is>
-          <t>Size (bp, if applicable)</t>
-        </is>
-      </c>
-      <c r="G43" s="97" t="inlineStr">
-        <is>
-          <t>i7 Index (if any)</t>
-        </is>
-      </c>
-      <c r="H43" s="98" t="inlineStr">
-        <is>
-          <t>i5 Index (NovaSeq 1.0/Forward)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="55" t="inlineStr">
-        <is>
-          <t>Example 1</t>
-        </is>
-      </c>
-      <c r="B44" s="93" t="n"/>
-      <c r="C44" s="93" t="n"/>
-      <c r="D44" s="93" t="n"/>
-      <c r="E44" s="93" t="n"/>
-      <c r="F44" s="93" t="n"/>
-      <c r="G44" s="93" t="n"/>
-      <c r="H44" s="94" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="55" t="inlineStr">
-        <is>
-          <t>Example 2</t>
-        </is>
-      </c>
-      <c r="B45" s="93" t="n"/>
-      <c r="C45" s="93" t="n"/>
-      <c r="D45" s="93" t="n"/>
-      <c r="E45" s="93" t="n"/>
-      <c r="F45" s="93" t="n"/>
-      <c r="G45" s="93" t="n"/>
-      <c r="H45" s="94" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="55" t="inlineStr">
-        <is>
-          <t>Example 3</t>
-        </is>
-      </c>
-      <c r="B46" s="93" t="n"/>
-      <c r="C46" s="93" t="n"/>
-      <c r="D46" s="93" t="n"/>
-      <c r="E46" s="93" t="n"/>
-      <c r="F46" s="93" t="n"/>
-      <c r="G46" s="93" t="n"/>
-      <c r="H46" s="94" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="55" t="inlineStr">
-        <is>
-          <t>Example 4</t>
-        </is>
-      </c>
-      <c r="B47" s="93" t="n"/>
-      <c r="C47" s="93" t="n"/>
-      <c r="D47" s="93" t="n"/>
-      <c r="E47" s="93" t="n"/>
-      <c r="F47" s="93" t="n"/>
-      <c r="G47" s="93" t="n"/>
-      <c r="H47" s="94" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="55" t="inlineStr">
-        <is>
-          <t>Example 5</t>
-        </is>
-      </c>
-      <c r="B48" s="93" t="n"/>
-      <c r="C48" s="93" t="n"/>
-      <c r="D48" s="93" t="n"/>
-      <c r="E48" s="93" t="n"/>
-      <c r="F48" s="93" t="n"/>
-      <c r="G48" s="93" t="n"/>
-      <c r="H48" s="94" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="55" t="inlineStr">
-        <is>
-          <t>Example 6</t>
-        </is>
-      </c>
-      <c r="B49" s="93" t="n"/>
-      <c r="C49" s="93" t="n"/>
-      <c r="D49" s="93" t="n"/>
-      <c r="E49" s="93" t="n"/>
-      <c r="F49" s="93" t="n"/>
-      <c r="G49" s="93" t="n"/>
-      <c r="H49" s="94" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="55" t="inlineStr">
-        <is>
-          <t>Example 7</t>
-        </is>
-      </c>
-      <c r="B50" s="93" t="n"/>
-      <c r="C50" s="93" t="n"/>
-      <c r="D50" s="93" t="n"/>
-      <c r="E50" s="93" t="n"/>
-      <c r="F50" s="93" t="n"/>
-      <c r="G50" s="93" t="n"/>
-      <c r="H50" s="94" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="55" t="inlineStr">
-        <is>
-          <t>Example 8</t>
-        </is>
-      </c>
-      <c r="B51" s="93" t="n"/>
-      <c r="C51" s="93" t="n"/>
-      <c r="D51" s="93" t="n"/>
-      <c r="E51" s="93" t="n"/>
-      <c r="F51" s="93" t="n"/>
-      <c r="G51" s="93" t="n"/>
-      <c r="H51" s="94" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="55" t="inlineStr">
-        <is>
-          <t>Example 9</t>
-        </is>
-      </c>
-      <c r="B52" s="93" t="n"/>
-      <c r="C52" s="93" t="n"/>
-      <c r="D52" s="93" t="n"/>
-      <c r="E52" s="93" t="n"/>
-      <c r="F52" s="93" t="n"/>
-      <c r="G52" s="93" t="n"/>
-      <c r="H52" s="94" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="59" t="inlineStr">
-        <is>
-          <t>Example 10</t>
-        </is>
-      </c>
-      <c r="B53" s="95" t="n"/>
-      <c r="C53" s="95" t="n"/>
-      <c r="D53" s="95" t="n"/>
-      <c r="E53" s="95" t="n"/>
-      <c r="F53" s="95" t="n"/>
-      <c r="G53" s="95" t="n"/>
-      <c r="H53" s="96" t="n"/>
+      <c r="B42" s="83" t="n"/>
+      <c r="C42" s="83" t="n"/>
+      <c r="D42" s="83" t="n"/>
+      <c r="E42" s="83" t="n"/>
+      <c r="F42" s="83" t="n"/>
+      <c r="G42" s="83" t="n"/>
+      <c r="H42" s="84" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
+  <mergeCells count="18">
     <mergeCell ref="A9:H9"/>
-    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B17:H17"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B5:H5"/>
     <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B10:H10"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="B11:H11"/>
     <mergeCell ref="B15:H15"/>
-    <mergeCell ref="B22:F22"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B21:F21"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B23:F23"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B28:F28"/>
-    <mergeCell ref="A42:H42"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B30:F30"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="A13:H13"/>
-    <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B19:H19"/>
-    <mergeCell ref="B26:F26"/>
   </mergeCells>
-  <dataValidations count="10">
-    <dataValidation sqref="F31:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+  <dataValidations count="9">
+    <dataValidation sqref="F20:F29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"4°C,Dry Ice"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="G31:G40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="G20:G29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Discard,Return,Extended Storage"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="H31:H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="H20:H29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B10:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="B10:H10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Mail,Drop Off,On Site (single cell only),Pick up (single cell only)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C44:C53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="C33:C42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Water,EB"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B31:B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="B20:B29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"RNA-Seq (mRNA),RNA-Seq (rRNA depletion),Single Cell (5'),Single Cell (3'),Single Cell (VDJ),Single Cell (5' + VDJ),Shotgun Meta,WGS,sequencing only"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="D31:D40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="D20:D29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Mouse,Human,Other (Please specify in Sample Note)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B44:B53" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="B33:B42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Total RNA,cDNA library"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C31:C40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="C20:C29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Body Fluid,Cell,Tissue,Whole Blood,Nucleic Acid,Stool,Water,Soil,cDNA Library"</formula1>
       <formula2>0</formula2>
-    </dataValidation>
-    <dataValidation sqref="G21:G30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Regular,Custom"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -1876,12 +1668,12 @@
       <c r="I1" s="65" t="n"/>
     </row>
     <row r="2" ht="43.5" customHeight="1" s="47">
-      <c r="A2" s="99" t="inlineStr">
+      <c r="A2" s="87" t="inlineStr">
         <is>
           <t>Mail</t>
         </is>
       </c>
-      <c r="B2" s="100" t="inlineStr">
+      <c r="B2" s="88" t="inlineStr">
         <is>
           <t>Please mail your samples to the following address: Jing Shi, Athenomics, 1 Grant St Suite 230, Framingham, MA, 01702 and fill the transportation company and tracking number in the Delivery Note.</t>
         </is>
@@ -1895,12 +1687,12 @@
       <c r="I2" s="54" t="n"/>
     </row>
     <row r="3" ht="27.75" customHeight="1" s="47">
-      <c r="A3" s="101" t="inlineStr">
+      <c r="A3" s="89" t="inlineStr">
         <is>
           <t>Dorp Off</t>
         </is>
       </c>
-      <c r="B3" s="102" t="inlineStr">
+      <c r="B3" s="90" t="inlineStr">
         <is>
           <t>Please fill in the expected the drop off time in the Delivery Note and text the operator at 4434538418 once drop off.</t>
         </is>
@@ -1914,38 +1706,38 @@
       <c r="I3" s="58" t="n"/>
     </row>
     <row r="4" ht="15" customHeight="1" s="47">
-      <c r="A4" s="103" t="inlineStr">
+      <c r="A4" s="91" t="inlineStr">
         <is>
           <t>On site</t>
         </is>
       </c>
-      <c r="B4" s="104" t="inlineStr">
+      <c r="B4" s="92" t="inlineStr">
         <is>
           <t>If pick up/on site is chosen, please fill in the expected the arrival time in the Delivery Note and settle down the details with operator before the scheduled time.</t>
         </is>
       </c>
-      <c r="C4" s="105" t="n"/>
-      <c r="D4" s="105" t="n"/>
-      <c r="E4" s="105" t="n"/>
-      <c r="F4" s="105" t="n"/>
-      <c r="G4" s="105" t="n"/>
-      <c r="H4" s="105" t="n"/>
-      <c r="I4" s="106" t="n"/>
+      <c r="C4" s="93" t="n"/>
+      <c r="D4" s="93" t="n"/>
+      <c r="E4" s="93" t="n"/>
+      <c r="F4" s="93" t="n"/>
+      <c r="G4" s="93" t="n"/>
+      <c r="H4" s="93" t="n"/>
+      <c r="I4" s="94" t="n"/>
     </row>
     <row r="5" ht="15" customHeight="1" s="47">
-      <c r="A5" s="107" t="inlineStr">
+      <c r="A5" s="95" t="inlineStr">
         <is>
           <t>Pick up</t>
         </is>
       </c>
-      <c r="B5" s="108" t="n"/>
-      <c r="C5" s="109" t="n"/>
-      <c r="D5" s="109" t="n"/>
-      <c r="E5" s="109" t="n"/>
-      <c r="F5" s="109" t="n"/>
-      <c r="G5" s="109" t="n"/>
-      <c r="H5" s="109" t="n"/>
-      <c r="I5" s="110" t="n"/>
+      <c r="B5" s="96" t="n"/>
+      <c r="C5" s="97" t="n"/>
+      <c r="D5" s="97" t="n"/>
+      <c r="E5" s="97" t="n"/>
+      <c r="F5" s="97" t="n"/>
+      <c r="G5" s="97" t="n"/>
+      <c r="H5" s="97" t="n"/>
+      <c r="I5" s="98" t="n"/>
     </row>
     <row r="6" ht="15" customHeight="1" s="47"/>
     <row r="7" ht="15" customHeight="1" s="47">
@@ -1964,12 +1756,12 @@
       <c r="I7" s="65" t="n"/>
     </row>
     <row r="8" ht="14.25" customHeight="1" s="47">
-      <c r="A8" s="111" t="inlineStr">
+      <c r="A8" s="99" t="inlineStr">
         <is>
           <t>bulk RNA transcriptome</t>
         </is>
       </c>
-      <c r="B8" s="112" t="inlineStr">
+      <c r="B8" s="100" t="inlineStr">
         <is>
           <t>Common animal or plant</t>
         </is>
@@ -2022,27 +1814,27 @@
     </row>
     <row r="11" ht="15" customHeight="1" s="47"/>
     <row r="12" ht="15" customHeight="1" s="47">
-      <c r="A12" s="113" t="inlineStr">
+      <c r="A12" s="101" t="inlineStr">
         <is>
           <t>Sample Requirement</t>
         </is>
       </c>
-      <c r="B12" s="114" t="n"/>
-      <c r="C12" s="114" t="n"/>
-      <c r="D12" s="114" t="n"/>
-      <c r="E12" s="114" t="n"/>
-      <c r="F12" s="114" t="n"/>
-      <c r="G12" s="114" t="n"/>
-      <c r="H12" s="114" t="n"/>
-      <c r="I12" s="115" t="n"/>
+      <c r="B12" s="102" t="n"/>
+      <c r="C12" s="102" t="n"/>
+      <c r="D12" s="102" t="n"/>
+      <c r="E12" s="102" t="n"/>
+      <c r="F12" s="102" t="n"/>
+      <c r="G12" s="102" t="n"/>
+      <c r="H12" s="102" t="n"/>
+      <c r="I12" s="103" t="n"/>
     </row>
     <row r="13" ht="45" customHeight="1" s="47">
-      <c r="A13" s="116" t="inlineStr">
+      <c r="A13" s="104" t="inlineStr">
         <is>
           <t>Body Fluid Sample:</t>
         </is>
       </c>
-      <c r="B13" s="100" t="inlineStr">
+      <c r="B13" s="88" t="inlineStr">
         <is>
           <t>Expected volume: 3mL. If to be mailed, mix with RNA Protect Reagent, ship at 4 degree within 2 days or ship with dry ice within 1 day. Drop off samples are recommended to be processed immediately before drop off and store at 4 degree or store in dry ice.</t>
         </is>
@@ -2056,12 +1848,12 @@
       <c r="I13" s="54" t="n"/>
     </row>
     <row r="14" ht="45" customHeight="1" s="47">
-      <c r="A14" s="117" t="inlineStr">
+      <c r="A14" s="105" t="inlineStr">
         <is>
           <t>Cell Sample:</t>
         </is>
       </c>
-      <c r="B14" s="102" t="inlineStr">
+      <c r="B14" s="90" t="inlineStr">
         <is>
           <t>Expected quantity: &gt;2E6 cells. If to be mailed, perserved with cell freezing media, ship with dry ice within 1 day. Drop off samples are recommended to be processed immediately before drop off and store at 4 degree or perserved with cell freezing media in dry ice.</t>
         </is>
@@ -2075,12 +1867,12 @@
       <c r="I14" s="58" t="n"/>
     </row>
     <row r="15" ht="30.75" customHeight="1" s="47">
-      <c r="A15" s="117" t="inlineStr">
+      <c r="A15" s="105" t="inlineStr">
         <is>
           <t>Tissue/Stool Sample:</t>
         </is>
       </c>
-      <c r="B15" s="102" t="inlineStr">
+      <c r="B15" s="90" t="inlineStr">
         <is>
           <t>Expected Mass: &gt;200mg, if to be mailed, ship with dry ice and within 1 day. Drop off samples are recommended to be processed immediately before drop off and store in dry ice.</t>
         </is>
@@ -2094,31 +1886,31 @@
       <c r="I15" s="58" t="n"/>
     </row>
     <row r="16" ht="14.25" customHeight="1" s="47">
-      <c r="A16" s="117" t="inlineStr">
+      <c r="A16" s="105" t="inlineStr">
         <is>
           <t>Whole Blood:</t>
         </is>
       </c>
-      <c r="B16" s="93" t="inlineStr">
+      <c r="B16" s="81" t="inlineStr">
         <is>
           <t>&gt;500µL Whole blood collected in EDTA tube immeidately before the arrival time, store at 4 degree</t>
         </is>
       </c>
-      <c r="C16" s="93" t="n"/>
-      <c r="D16" s="93" t="n"/>
-      <c r="E16" s="93" t="n"/>
-      <c r="F16" s="93" t="n"/>
-      <c r="G16" s="93" t="n"/>
-      <c r="H16" s="93" t="n"/>
-      <c r="I16" s="94" t="n"/>
+      <c r="C16" s="81" t="n"/>
+      <c r="D16" s="81" t="n"/>
+      <c r="E16" s="81" t="n"/>
+      <c r="F16" s="81" t="n"/>
+      <c r="G16" s="81" t="n"/>
+      <c r="H16" s="81" t="n"/>
+      <c r="I16" s="82" t="n"/>
     </row>
     <row r="17" ht="30" customHeight="1" s="47">
-      <c r="A17" s="117" t="inlineStr">
+      <c r="A17" s="105" t="inlineStr">
         <is>
           <t>Total RNA/genomic DNA:</t>
         </is>
       </c>
-      <c r="B17" s="102" t="inlineStr">
+      <c r="B17" s="90" t="inlineStr">
         <is>
           <t>Expected quantity: 2µg - 10µg, 20µL - 50µL. If to be mailed, ship with dry ice within 1 day. Drop off samples are recommended to be stored in dry ice.</t>
         </is>
@@ -2132,12 +1924,12 @@
       <c r="I17" s="58" t="n"/>
     </row>
     <row r="18" ht="30.75" customHeight="1" s="47">
-      <c r="A18" s="117" t="inlineStr">
+      <c r="A18" s="105" t="inlineStr">
         <is>
           <t>cDNA Library:</t>
         </is>
       </c>
-      <c r="B18" s="102" t="inlineStr">
+      <c r="B18" s="90" t="inlineStr">
         <is>
           <t>Expected quantity: &gt;200ng in at least 10µL. If to be mailed, ship with dry ice within 1 day. Drop off samples are recommended to be stored in dry ice.</t>
         </is>
@@ -2151,12 +1943,12 @@
       <c r="I18" s="58" t="n"/>
     </row>
     <row r="19" ht="45.75" customHeight="1" s="47">
-      <c r="A19" s="117" t="inlineStr">
+      <c r="A19" s="105" t="inlineStr">
         <is>
           <t>Water Sample:</t>
         </is>
       </c>
-      <c r="B19" s="102" t="inlineStr">
+      <c r="B19" s="90" t="inlineStr">
         <is>
           <t>Expected volume: 3mL. If to be mailed, ship at 4 degree within 2 days or ship with dry ice within 1 day. Drop off samples are recommended to be processed immediately before drop off and store at 4 degree or store in dry ice.</t>
         </is>
@@ -2170,12 +1962,12 @@
       <c r="I19" s="58" t="n"/>
     </row>
     <row r="20" ht="45" customHeight="1" s="47">
-      <c r="A20" s="118" t="inlineStr">
+      <c r="A20" s="106" t="inlineStr">
         <is>
           <t>Soil Sample:</t>
         </is>
       </c>
-      <c r="B20" s="104" t="inlineStr">
+      <c r="B20" s="92" t="inlineStr">
         <is>
           <t>Expected Mass: &gt;1g. If to be mailed, ship at 4 degree within 2 days or ship with dry ice within 1 day. Drop off samples are recommended to be processed immediately before drop off and store at 4 degree or store in dry ice.</t>
         </is>
@@ -2205,12 +1997,12 @@
       <c r="I22" s="65" t="n"/>
     </row>
     <row r="23" ht="28.5" customHeight="1" s="47">
-      <c r="A23" s="119" t="inlineStr">
+      <c r="A23" s="107" t="inlineStr">
         <is>
           <t>Default Sample Storage Time</t>
         </is>
       </c>
-      <c r="B23" s="100" t="inlineStr">
+      <c r="B23" s="88" t="inlineStr">
         <is>
           <t>1 Month (Return or extended storage are available with additional charge. Return charge: $150. Storage charge: $0.2/per sample/per month.)</t>
         </is>
@@ -2224,12 +2016,12 @@
       <c r="I23" s="54" t="n"/>
     </row>
     <row r="24" ht="30" customHeight="1" s="47">
-      <c r="A24" s="120" t="inlineStr">
+      <c r="A24" s="108" t="inlineStr">
         <is>
           <t>Default Data Storage Time</t>
         </is>
       </c>
-      <c r="B24" s="104" t="inlineStr">
+      <c r="B24" s="92" t="inlineStr">
         <is>
           <t>2 Months (Extended storage are available with additional charge. Storage charge: $0.1/G/per month.)</t>
         </is>
@@ -2247,8 +2039,8 @@
     <mergeCell ref="B4:I5"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B9:I9"/>
     <mergeCell ref="B18:I18"/>
-    <mergeCell ref="B9:I9"/>
     <mergeCell ref="B15:I15"/>
     <mergeCell ref="B24:I24"/>
     <mergeCell ref="B2:I2"/>

</xml_diff>

<commit_message>
rewrite rows 15-19 text + insert Per-Sample Details divider row
Add default-method-if-unspecified clause; visually separate overall
submission info (15-19) from per-sample table (20+, shifted by 1).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
+++ b/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
@@ -372,7 +372,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="110">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -661,6 +661,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -929,7 +932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38.44" customWidth="1" style="46" min="1" max="1"/>
@@ -1120,7 +1123,8 @@
       </c>
       <c r="B15" s="73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please read the following instruction, then delete all the default/sample and input your information and instruction  </t>
+          <t>Please read the following instructions, then delete all the default/sample text and input your own information and instructions.
+This section (rows 15-19) is your OVERALL submission information — what you want analyzed and how. Individual sample details go in the table below (see the "Per-Sample Details" section).</t>
         </is>
       </c>
       <c r="C15" s="64" t="n"/>
@@ -1138,8 +1142,9 @@
       </c>
       <c r="B16" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Please specify the source of sample as detail as possible at here, such as 
-Cell line, organ, tissue, iPSCs, humanized mice, human cells expressed in mice ,  tumor/normal ,  stool , blood, brain etc. </t>
+          <t>Please specify the source of sample in general, as detail as possible, such as 
+Cell line, organ, tissue, iPSCs, humanized mice, human cells expressed in mice, tumor/normal, stool, blood, brain etc.
+(This is the overall/general sample description for the whole submission — the type, species, and storage condition of each individual sample are recorded in the Per-Sample Details table below.)</t>
         </is>
       </c>
       <c r="C16" s="64" t="n"/>
@@ -1197,7 +1202,7 @@
       <c r="G18" s="64" t="n"/>
       <c r="H18" s="65" t="n"/>
     </row>
-    <row r="19" ht="210" customHeight="1" s="47">
+    <row r="19" ht="260" customHeight="1" s="47">
       <c r="A19" s="79" t="inlineStr">
         <is>
           <t>Analysis requirements:
@@ -1216,7 +1221,14 @@
 and Setting field above, will NOT be
 included in the analysis or the quote
 unless this form is updated and
-re-submitted.</t>
+re-submitted.
+ℹ If you do NOT specify a particular
+detail (e.g. a filtering threshold,
+statistical test, or significance cutoff),
+our analyst will apply the company's
+default / current statistical best-practice
+method for that analysis type, and will
+state the choice made in the final report.</t>
         </is>
       </c>
       <c r="B19" s="80" t="inlineStr">
@@ -1237,24 +1249,24 @@
       <c r="G19" s="64" t="n"/>
       <c r="H19" s="65" t="n"/>
     </row>
-    <row r="20" ht="15" customHeight="1" s="47">
-      <c r="A20" s="55" t="inlineStr">
-        <is>
-          <t>Example 1</t>
-        </is>
-      </c>
-      <c r="B20" s="81" t="n"/>
-      <c r="C20" s="81" t="n"/>
-      <c r="D20" s="81" t="n"/>
-      <c r="E20" s="81" t="n"/>
-      <c r="F20" s="81" t="n"/>
-      <c r="G20" s="81" t="n"/>
-      <c r="H20" s="82" t="n"/>
+    <row r="20" ht="32" customHeight="1" s="47">
+      <c r="A20" s="109" t="inlineStr">
+        <is>
+          <t>▼ PER-SAMPLE DETAILS (below) — one row per individual physical sample.  The section above (rows 15-19) covers your overall submission: sample description, analysis type, and requirements.</t>
+        </is>
+      </c>
+      <c r="B20" s="64" t="n"/>
+      <c r="C20" s="64" t="n"/>
+      <c r="D20" s="64" t="n"/>
+      <c r="E20" s="64" t="n"/>
+      <c r="F20" s="64" t="n"/>
+      <c r="G20" s="64" t="n"/>
+      <c r="H20" s="65" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="47">
       <c r="A21" s="55" t="inlineStr">
         <is>
-          <t>Example 2</t>
+          <t>Example 1</t>
         </is>
       </c>
       <c r="B21" s="81" t="n"/>
@@ -1268,7 +1280,7 @@
     <row r="22" ht="15" customHeight="1" s="47">
       <c r="A22" s="55" t="inlineStr">
         <is>
-          <t>Example 3</t>
+          <t>Example 2</t>
         </is>
       </c>
       <c r="B22" s="81" t="n"/>
@@ -1282,7 +1294,7 @@
     <row r="23" ht="15" customHeight="1" s="47">
       <c r="A23" s="55" t="inlineStr">
         <is>
-          <t>Example 4</t>
+          <t>Example 3</t>
         </is>
       </c>
       <c r="B23" s="81" t="n"/>
@@ -1296,7 +1308,7 @@
     <row r="24" ht="15" customHeight="1" s="47">
       <c r="A24" s="55" t="inlineStr">
         <is>
-          <t>Example 5</t>
+          <t>Example 4</t>
         </is>
       </c>
       <c r="B24" s="81" t="n"/>
@@ -1310,7 +1322,7 @@
     <row r="25" ht="15" customHeight="1" s="47">
       <c r="A25" s="55" t="inlineStr">
         <is>
-          <t>Example 6</t>
+          <t>Example 5</t>
         </is>
       </c>
       <c r="B25" s="81" t="n"/>
@@ -1324,7 +1336,7 @@
     <row r="26" ht="15" customHeight="1" s="47">
       <c r="A26" s="55" t="inlineStr">
         <is>
-          <t>Example 7</t>
+          <t>Example 6</t>
         </is>
       </c>
       <c r="B26" s="81" t="n"/>
@@ -1338,7 +1350,7 @@
     <row r="27" ht="15" customHeight="1" s="47">
       <c r="A27" s="55" t="inlineStr">
         <is>
-          <t>Example 8</t>
+          <t>Example 7</t>
         </is>
       </c>
       <c r="B27" s="81" t="n"/>
@@ -1352,7 +1364,7 @@
     <row r="28" ht="15" customHeight="1" s="47">
       <c r="A28" s="55" t="inlineStr">
         <is>
-          <t>Example 9</t>
+          <t>Example 8</t>
         </is>
       </c>
       <c r="B28" s="81" t="n"/>
@@ -1364,94 +1376,94 @@
       <c r="H28" s="82" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="47">
-      <c r="A29" s="59" t="inlineStr">
+      <c r="A29" s="55" t="inlineStr">
+        <is>
+          <t>Example 9</t>
+        </is>
+      </c>
+      <c r="B29" s="81" t="n"/>
+      <c r="C29" s="81" t="n"/>
+      <c r="D29" s="81" t="n"/>
+      <c r="E29" s="81" t="n"/>
+      <c r="F29" s="81" t="n"/>
+      <c r="G29" s="81" t="n"/>
+      <c r="H29" s="82" t="n"/>
+    </row>
+    <row r="30" ht="15" customHeight="1" s="47">
+      <c r="A30" s="59" t="inlineStr">
         <is>
           <t>Example 10</t>
         </is>
       </c>
-      <c r="B29" s="83" t="n"/>
-      <c r="C29" s="83" t="n"/>
-      <c r="D29" s="83" t="n"/>
-      <c r="E29" s="83" t="n"/>
-      <c r="F29" s="83" t="n"/>
-      <c r="G29" s="83" t="n"/>
-      <c r="H29" s="84" t="n"/>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="47"/>
-    <row r="31" ht="15" customHeight="1" s="47">
-      <c r="A31" s="63" t="inlineStr">
+      <c r="B30" s="83" t="n"/>
+      <c r="C30" s="83" t="n"/>
+      <c r="D30" s="83" t="n"/>
+      <c r="E30" s="83" t="n"/>
+      <c r="F30" s="83" t="n"/>
+      <c r="G30" s="83" t="n"/>
+      <c r="H30" s="84" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="47"/>
+    <row r="32" ht="14.25" customHeight="1" s="47">
+      <c r="A32" s="63" t="inlineStr">
         <is>
           <t>Nucleic Acids Additional Information</t>
         </is>
       </c>
-      <c r="B31" s="64" t="n"/>
-      <c r="C31" s="64" t="n"/>
-      <c r="D31" s="64" t="n"/>
-      <c r="E31" s="64" t="n"/>
-      <c r="F31" s="64" t="n"/>
-      <c r="G31" s="64" t="n"/>
-      <c r="H31" s="65" t="n"/>
-    </row>
-    <row r="32" ht="14.25" customHeight="1" s="47">
-      <c r="A32" s="66" t="inlineStr">
+      <c r="B32" s="64" t="n"/>
+      <c r="C32" s="64" t="n"/>
+      <c r="D32" s="64" t="n"/>
+      <c r="E32" s="64" t="n"/>
+      <c r="F32" s="64" t="n"/>
+      <c r="G32" s="64" t="n"/>
+      <c r="H32" s="65" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="47">
+      <c r="A33" s="66" t="inlineStr">
         <is>
           <t>Sample Name</t>
         </is>
       </c>
-      <c r="B32" s="85" t="inlineStr">
+      <c r="B33" s="85" t="inlineStr">
         <is>
           <t>Nucleic Acid Type</t>
         </is>
       </c>
-      <c r="C32" s="85" t="inlineStr">
+      <c r="C33" s="85" t="inlineStr">
         <is>
           <t>Storage Reagent</t>
         </is>
       </c>
-      <c r="D32" s="85" t="inlineStr">
+      <c r="D33" s="85" t="inlineStr">
         <is>
           <t>Concentration (ng/µL)</t>
         </is>
       </c>
-      <c r="E32" s="85" t="inlineStr">
+      <c r="E33" s="85" t="inlineStr">
         <is>
           <t>Volume (µL)</t>
         </is>
       </c>
-      <c r="F32" s="85" t="inlineStr">
+      <c r="F33" s="85" t="inlineStr">
         <is>
           <t>Size (bp, if applicable)</t>
         </is>
       </c>
-      <c r="G32" s="85" t="inlineStr">
+      <c r="G33" s="85" t="inlineStr">
         <is>
           <t>i7 Index (if any)</t>
         </is>
       </c>
-      <c r="H32" s="86" t="inlineStr">
+      <c r="H33" s="86" t="inlineStr">
         <is>
           <t>i5 Index (NovaSeq 1.0/Forward)</t>
         </is>
       </c>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="47">
-      <c r="A33" s="55" t="inlineStr">
-        <is>
-          <t>Example 1</t>
-        </is>
-      </c>
-      <c r="B33" s="81" t="n"/>
-      <c r="C33" s="81" t="n"/>
-      <c r="D33" s="81" t="n"/>
-      <c r="E33" s="81" t="n"/>
-      <c r="F33" s="81" t="n"/>
-      <c r="G33" s="81" t="n"/>
-      <c r="H33" s="82" t="n"/>
     </row>
     <row r="34" ht="15" customHeight="1" s="47">
       <c r="A34" s="55" t="inlineStr">
         <is>
-          <t>Example 2</t>
+          <t>Example 1</t>
         </is>
       </c>
       <c r="B34" s="81" t="n"/>
@@ -1465,7 +1477,7 @@
     <row r="35" ht="14.25" customHeight="1" s="47">
       <c r="A35" s="55" t="inlineStr">
         <is>
-          <t>Example 3</t>
+          <t>Example 2</t>
         </is>
       </c>
       <c r="B35" s="81" t="n"/>
@@ -1479,7 +1491,7 @@
     <row r="36" ht="14.25" customHeight="1" s="47">
       <c r="A36" s="55" t="inlineStr">
         <is>
-          <t>Example 4</t>
+          <t>Example 3</t>
         </is>
       </c>
       <c r="B36" s="81" t="n"/>
@@ -1493,7 +1505,7 @@
     <row r="37" ht="14.25" customHeight="1" s="47">
       <c r="A37" s="55" t="inlineStr">
         <is>
-          <t>Example 5</t>
+          <t>Example 4</t>
         </is>
       </c>
       <c r="B37" s="81" t="n"/>
@@ -1507,7 +1519,7 @@
     <row r="38" ht="14.25" customHeight="1" s="47">
       <c r="A38" s="55" t="inlineStr">
         <is>
-          <t>Example 6</t>
+          <t>Example 5</t>
         </is>
       </c>
       <c r="B38" s="81" t="n"/>
@@ -1521,7 +1533,7 @@
     <row r="39" ht="14.25" customHeight="1" s="47">
       <c r="A39" s="55" t="inlineStr">
         <is>
-          <t>Example 7</t>
+          <t>Example 6</t>
         </is>
       </c>
       <c r="B39" s="81" t="n"/>
@@ -1535,7 +1547,7 @@
     <row r="40" ht="14.25" customHeight="1" s="47">
       <c r="A40" s="55" t="inlineStr">
         <is>
-          <t>Example 8</t>
+          <t>Example 7</t>
         </is>
       </c>
       <c r="B40" s="81" t="n"/>
@@ -1549,7 +1561,7 @@
     <row r="41" ht="14.25" customHeight="1" s="47">
       <c r="A41" s="55" t="inlineStr">
         <is>
-          <t>Example 9</t>
+          <t>Example 8</t>
         </is>
       </c>
       <c r="B41" s="81" t="n"/>
@@ -1561,74 +1573,89 @@
       <c r="H41" s="82" t="n"/>
     </row>
     <row r="42" ht="15" customHeight="1" s="47">
-      <c r="A42" s="59" t="inlineStr">
+      <c r="A42" s="55" t="inlineStr">
+        <is>
+          <t>Example 9</t>
+        </is>
+      </c>
+      <c r="B42" s="81" t="n"/>
+      <c r="C42" s="81" t="n"/>
+      <c r="D42" s="81" t="n"/>
+      <c r="E42" s="81" t="n"/>
+      <c r="F42" s="81" t="n"/>
+      <c r="G42" s="81" t="n"/>
+      <c r="H42" s="82" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="59" t="inlineStr">
         <is>
           <t>Example 10</t>
         </is>
       </c>
-      <c r="B42" s="83" t="n"/>
-      <c r="C42" s="83" t="n"/>
-      <c r="D42" s="83" t="n"/>
-      <c r="E42" s="83" t="n"/>
-      <c r="F42" s="83" t="n"/>
-      <c r="G42" s="83" t="n"/>
-      <c r="H42" s="84" t="n"/>
+      <c r="B43" s="83" t="n"/>
+      <c r="C43" s="83" t="n"/>
+      <c r="D43" s="83" t="n"/>
+      <c r="E43" s="83" t="n"/>
+      <c r="F43" s="83" t="n"/>
+      <c r="G43" s="83" t="n"/>
+      <c r="H43" s="84" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="19">
     <mergeCell ref="A9:H9"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="B15:H15"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B7:H7"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B18:H18"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="B11:H11"/>
+    <mergeCell ref="A32:H32"/>
     <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B18:H18"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B5:H5"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A14:H14"/>
-    <mergeCell ref="B7:H7"/>
     <mergeCell ref="B10:H10"/>
-    <mergeCell ref="B3:H3"/>
     <mergeCell ref="B19:H19"/>
-    <mergeCell ref="A31:H31"/>
-    <mergeCell ref="B11:H11"/>
-    <mergeCell ref="B15:H15"/>
   </mergeCells>
   <dataValidations count="9">
-    <dataValidation sqref="F20:F29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="F21:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"4°C,Dry Ice"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="G20:G29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="G21:G30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Discard,Return,Extended Storage"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="H20:H29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="H21:H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B10:H10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="B10:H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Mail,Drop Off,On Site (single cell only),Pick up (single cell only)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C33:C42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="C34:C43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Water,EB"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B20:B29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="B21:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"RNA-Seq (mRNA),RNA-Seq (rRNA depletion),Single Cell (5'),Single Cell (3'),Single Cell (VDJ),Single Cell (5' + VDJ),Shotgun Meta,WGS,sequencing only"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="D20:D29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="D21:D30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Mouse,Human,Other (Please specify in Sample Note)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B33:B42" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="B34:B43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Total RNA,cDNA library"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C20:C29" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="C21:C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Body Fluid,Cell,Tissue,Whole Blood,Nucleic Acid,Stool,Water,Soil,cDNA Library"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -2039,8 +2066,8 @@
     <mergeCell ref="B4:I5"/>
     <mergeCell ref="A7:I7"/>
     <mergeCell ref="B13:I13"/>
+    <mergeCell ref="B18:I18"/>
     <mergeCell ref="B9:I9"/>
-    <mergeCell ref="B18:I18"/>
     <mergeCell ref="B15:I15"/>
     <mergeCell ref="B24:I24"/>
     <mergeCell ref="B2:I2"/>

</xml_diff>

<commit_message>
split Important pricing-basis notice into its own row above row 19
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
+++ b/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -92,6 +92,7 @@
       <color theme="1"/>
       <sz val="11"/>
     </font>
+    <font/>
   </fonts>
   <fills count="2">
     <fill>
@@ -101,7 +102,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="38">
     <border>
       <left/>
       <right/>
@@ -361,6 +362,7 @@
       <bottom style="medium"/>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -932,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38.44" customWidth="1" style="46" min="1" max="1"/>
@@ -1202,17 +1204,16 @@
       <c r="G18" s="64" t="n"/>
       <c r="H18" s="65" t="n"/>
     </row>
-    <row r="19" ht="260" customHeight="1" s="47">
+    <row r="19" ht="95" customHeight="1" s="47">
       <c r="A19" s="79" t="inlineStr">
         <is>
-          <t>Analysis requirements:
-Regular work for your selected category
-have no extra fee.
-Custom requirements has Additional fee
-($120/h).
-Our specialist will tell you which one is
-Custom item.
-⚠ IMPORTANT: This form — Sample Note +
+          <t>⚠ IMPORTANT
+(pricing basis)</t>
+        </is>
+      </c>
+      <c r="B19" s="80" t="inlineStr">
+        <is>
+          <t>⚠ IMPORTANT: This form — Sample Note +
 Analysis Type + Analysis Purpose and
 Setting above — is the SOLE basis for
 analysis scope and pricing. Requirements
@@ -1221,7 +1222,20 @@
 and Setting field above, will NOT be
 included in the analysis or the quote
 unless this form is updated and
-re-submitted.
+re-submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="165" customHeight="1" s="47">
+      <c r="A20" s="79" t="inlineStr">
+        <is>
+          <t>Analysis requirements:
+Regular work for your selected category
+have no extra fee.
+Custom requirements has Additional fee
+($120/h).
+Our specialist will tell you which one is
+Custom item.
 ℹ If you do NOT specify a particular
 detail (e.g. a filtering threshold,
 statistical test, or significance cutoff),
@@ -1231,7 +1245,7 @@
 state the choice made in the final report.</t>
         </is>
       </c>
-      <c r="B19" s="80" t="inlineStr">
+      <c r="B20" s="80" t="inlineStr">
         <is>
           <t>For example, the following item is regular items for wgs : 
 * Call germline short variants (SNV/indel) genome-wide and annotate them for population rarity (gnomAD) and clinical significance (ClinVar).
@@ -1242,20 +1256,6 @@
 * Perform HLA genotyping (class I and class II) from the WGS data.</t>
         </is>
       </c>
-      <c r="C19" s="64" t="n"/>
-      <c r="D19" s="64" t="n"/>
-      <c r="E19" s="64" t="n"/>
-      <c r="F19" s="64" t="n"/>
-      <c r="G19" s="64" t="n"/>
-      <c r="H19" s="65" t="n"/>
-    </row>
-    <row r="20" ht="32" customHeight="1" s="47">
-      <c r="A20" s="109" t="inlineStr">
-        <is>
-          <t>▼ PER-SAMPLE DETAILS (below) — one row per individual physical sample.  The section above (rows 15-19) covers your overall submission: sample description, analysis type, and requirements.</t>
-        </is>
-      </c>
-      <c r="B20" s="64" t="n"/>
       <c r="C20" s="64" t="n"/>
       <c r="D20" s="64" t="n"/>
       <c r="E20" s="64" t="n"/>
@@ -1263,24 +1263,24 @@
       <c r="G20" s="64" t="n"/>
       <c r="H20" s="65" t="n"/>
     </row>
-    <row r="21" ht="15" customHeight="1" s="47">
-      <c r="A21" s="55" t="inlineStr">
-        <is>
-          <t>Example 1</t>
-        </is>
-      </c>
-      <c r="B21" s="81" t="n"/>
-      <c r="C21" s="81" t="n"/>
-      <c r="D21" s="81" t="n"/>
-      <c r="E21" s="81" t="n"/>
-      <c r="F21" s="81" t="n"/>
-      <c r="G21" s="81" t="n"/>
-      <c r="H21" s="82" t="n"/>
+    <row r="21" ht="32" customHeight="1" s="47">
+      <c r="A21" s="109" t="inlineStr">
+        <is>
+          <t>▼ PER-SAMPLE DETAILS (below) — one row per individual physical sample.  The section above (rows 15-19) covers your overall submission: sample description, analysis type, and requirements.</t>
+        </is>
+      </c>
+      <c r="B21" s="64" t="n"/>
+      <c r="C21" s="64" t="n"/>
+      <c r="D21" s="64" t="n"/>
+      <c r="E21" s="64" t="n"/>
+      <c r="F21" s="64" t="n"/>
+      <c r="G21" s="64" t="n"/>
+      <c r="H21" s="65" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="47">
       <c r="A22" s="55" t="inlineStr">
         <is>
-          <t>Example 2</t>
+          <t>Example 1</t>
         </is>
       </c>
       <c r="B22" s="81" t="n"/>
@@ -1294,7 +1294,7 @@
     <row r="23" ht="15" customHeight="1" s="47">
       <c r="A23" s="55" t="inlineStr">
         <is>
-          <t>Example 3</t>
+          <t>Example 2</t>
         </is>
       </c>
       <c r="B23" s="81" t="n"/>
@@ -1308,7 +1308,7 @@
     <row r="24" ht="15" customHeight="1" s="47">
       <c r="A24" s="55" t="inlineStr">
         <is>
-          <t>Example 4</t>
+          <t>Example 3</t>
         </is>
       </c>
       <c r="B24" s="81" t="n"/>
@@ -1322,7 +1322,7 @@
     <row r="25" ht="15" customHeight="1" s="47">
       <c r="A25" s="55" t="inlineStr">
         <is>
-          <t>Example 5</t>
+          <t>Example 4</t>
         </is>
       </c>
       <c r="B25" s="81" t="n"/>
@@ -1336,7 +1336,7 @@
     <row r="26" ht="15" customHeight="1" s="47">
       <c r="A26" s="55" t="inlineStr">
         <is>
-          <t>Example 6</t>
+          <t>Example 5</t>
         </is>
       </c>
       <c r="B26" s="81" t="n"/>
@@ -1350,7 +1350,7 @@
     <row r="27" ht="15" customHeight="1" s="47">
       <c r="A27" s="55" t="inlineStr">
         <is>
-          <t>Example 7</t>
+          <t>Example 6</t>
         </is>
       </c>
       <c r="B27" s="81" t="n"/>
@@ -1364,7 +1364,7 @@
     <row r="28" ht="15" customHeight="1" s="47">
       <c r="A28" s="55" t="inlineStr">
         <is>
-          <t>Example 8</t>
+          <t>Example 7</t>
         </is>
       </c>
       <c r="B28" s="81" t="n"/>
@@ -1378,7 +1378,7 @@
     <row r="29" ht="15" customHeight="1" s="47">
       <c r="A29" s="55" t="inlineStr">
         <is>
-          <t>Example 9</t>
+          <t>Example 8</t>
         </is>
       </c>
       <c r="B29" s="81" t="n"/>
@@ -1390,94 +1390,94 @@
       <c r="H29" s="82" t="n"/>
     </row>
     <row r="30" ht="15" customHeight="1" s="47">
-      <c r="A30" s="59" t="inlineStr">
+      <c r="A30" s="55" t="inlineStr">
+        <is>
+          <t>Example 9</t>
+        </is>
+      </c>
+      <c r="B30" s="81" t="n"/>
+      <c r="C30" s="81" t="n"/>
+      <c r="D30" s="81" t="n"/>
+      <c r="E30" s="81" t="n"/>
+      <c r="F30" s="81" t="n"/>
+      <c r="G30" s="81" t="n"/>
+      <c r="H30" s="82" t="n"/>
+    </row>
+    <row r="31" ht="15" customHeight="1" s="47">
+      <c r="A31" s="59" t="inlineStr">
         <is>
           <t>Example 10</t>
         </is>
       </c>
-      <c r="B30" s="83" t="n"/>
-      <c r="C30" s="83" t="n"/>
-      <c r="D30" s="83" t="n"/>
-      <c r="E30" s="83" t="n"/>
-      <c r="F30" s="83" t="n"/>
-      <c r="G30" s="83" t="n"/>
-      <c r="H30" s="84" t="n"/>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="47"/>
-    <row r="32" ht="14.25" customHeight="1" s="47">
-      <c r="A32" s="63" t="inlineStr">
+      <c r="B31" s="83" t="n"/>
+      <c r="C31" s="83" t="n"/>
+      <c r="D31" s="83" t="n"/>
+      <c r="E31" s="83" t="n"/>
+      <c r="F31" s="83" t="n"/>
+      <c r="G31" s="83" t="n"/>
+      <c r="H31" s="84" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="47"/>
+    <row r="33" ht="14.25" customHeight="1" s="47">
+      <c r="A33" s="63" t="inlineStr">
         <is>
           <t>Nucleic Acids Additional Information</t>
         </is>
       </c>
-      <c r="B32" s="64" t="n"/>
-      <c r="C32" s="64" t="n"/>
-      <c r="D32" s="64" t="n"/>
-      <c r="E32" s="64" t="n"/>
-      <c r="F32" s="64" t="n"/>
-      <c r="G32" s="64" t="n"/>
-      <c r="H32" s="65" t="n"/>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="47">
-      <c r="A33" s="66" t="inlineStr">
+      <c r="B33" s="64" t="n"/>
+      <c r="C33" s="64" t="n"/>
+      <c r="D33" s="64" t="n"/>
+      <c r="E33" s="64" t="n"/>
+      <c r="F33" s="64" t="n"/>
+      <c r="G33" s="64" t="n"/>
+      <c r="H33" s="65" t="n"/>
+    </row>
+    <row r="34" ht="15" customHeight="1" s="47">
+      <c r="A34" s="66" t="inlineStr">
         <is>
           <t>Sample Name</t>
         </is>
       </c>
-      <c r="B33" s="85" t="inlineStr">
+      <c r="B34" s="85" t="inlineStr">
         <is>
           <t>Nucleic Acid Type</t>
         </is>
       </c>
-      <c r="C33" s="85" t="inlineStr">
+      <c r="C34" s="85" t="inlineStr">
         <is>
           <t>Storage Reagent</t>
         </is>
       </c>
-      <c r="D33" s="85" t="inlineStr">
+      <c r="D34" s="85" t="inlineStr">
         <is>
           <t>Concentration (ng/µL)</t>
         </is>
       </c>
-      <c r="E33" s="85" t="inlineStr">
+      <c r="E34" s="85" t="inlineStr">
         <is>
           <t>Volume (µL)</t>
         </is>
       </c>
-      <c r="F33" s="85" t="inlineStr">
+      <c r="F34" s="85" t="inlineStr">
         <is>
           <t>Size (bp, if applicable)</t>
         </is>
       </c>
-      <c r="G33" s="85" t="inlineStr">
+      <c r="G34" s="85" t="inlineStr">
         <is>
           <t>i7 Index (if any)</t>
         </is>
       </c>
-      <c r="H33" s="86" t="inlineStr">
+      <c r="H34" s="86" t="inlineStr">
         <is>
           <t>i5 Index (NovaSeq 1.0/Forward)</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="47">
-      <c r="A34" s="55" t="inlineStr">
+    <row r="35" ht="15" customHeight="1" s="47">
+      <c r="A35" s="55" t="inlineStr">
         <is>
           <t>Example 1</t>
-        </is>
-      </c>
-      <c r="B34" s="81" t="n"/>
-      <c r="C34" s="81" t="n"/>
-      <c r="D34" s="81" t="n"/>
-      <c r="E34" s="81" t="n"/>
-      <c r="F34" s="81" t="n"/>
-      <c r="G34" s="81" t="n"/>
-      <c r="H34" s="82" t="n"/>
-    </row>
-    <row r="35" ht="14.25" customHeight="1" s="47">
-      <c r="A35" s="55" t="inlineStr">
-        <is>
-          <t>Example 2</t>
         </is>
       </c>
       <c r="B35" s="81" t="n"/>
@@ -1491,7 +1491,7 @@
     <row r="36" ht="14.25" customHeight="1" s="47">
       <c r="A36" s="55" t="inlineStr">
         <is>
-          <t>Example 3</t>
+          <t>Example 2</t>
         </is>
       </c>
       <c r="B36" s="81" t="n"/>
@@ -1505,7 +1505,7 @@
     <row r="37" ht="14.25" customHeight="1" s="47">
       <c r="A37" s="55" t="inlineStr">
         <is>
-          <t>Example 4</t>
+          <t>Example 3</t>
         </is>
       </c>
       <c r="B37" s="81" t="n"/>
@@ -1519,7 +1519,7 @@
     <row r="38" ht="14.25" customHeight="1" s="47">
       <c r="A38" s="55" t="inlineStr">
         <is>
-          <t>Example 5</t>
+          <t>Example 4</t>
         </is>
       </c>
       <c r="B38" s="81" t="n"/>
@@ -1533,7 +1533,7 @@
     <row r="39" ht="14.25" customHeight="1" s="47">
       <c r="A39" s="55" t="inlineStr">
         <is>
-          <t>Example 6</t>
+          <t>Example 5</t>
         </is>
       </c>
       <c r="B39" s="81" t="n"/>
@@ -1547,7 +1547,7 @@
     <row r="40" ht="14.25" customHeight="1" s="47">
       <c r="A40" s="55" t="inlineStr">
         <is>
-          <t>Example 7</t>
+          <t>Example 6</t>
         </is>
       </c>
       <c r="B40" s="81" t="n"/>
@@ -1561,7 +1561,7 @@
     <row r="41" ht="14.25" customHeight="1" s="47">
       <c r="A41" s="55" t="inlineStr">
         <is>
-          <t>Example 8</t>
+          <t>Example 7</t>
         </is>
       </c>
       <c r="B41" s="81" t="n"/>
@@ -1572,10 +1572,10 @@
       <c r="G41" s="81" t="n"/>
       <c r="H41" s="82" t="n"/>
     </row>
-    <row r="42" ht="15" customHeight="1" s="47">
+    <row r="42" ht="14.25" customHeight="1" s="47">
       <c r="A42" s="55" t="inlineStr">
         <is>
-          <t>Example 9</t>
+          <t>Example 8</t>
         </is>
       </c>
       <c r="B42" s="81" t="n"/>
@@ -1586,52 +1586,67 @@
       <c r="G42" s="81" t="n"/>
       <c r="H42" s="82" t="n"/>
     </row>
-    <row r="43">
-      <c r="A43" s="59" t="inlineStr">
+    <row r="43" ht="15" customHeight="1" s="47">
+      <c r="A43" s="55" t="inlineStr">
+        <is>
+          <t>Example 9</t>
+        </is>
+      </c>
+      <c r="B43" s="81" t="n"/>
+      <c r="C43" s="81" t="n"/>
+      <c r="D43" s="81" t="n"/>
+      <c r="E43" s="81" t="n"/>
+      <c r="F43" s="81" t="n"/>
+      <c r="G43" s="81" t="n"/>
+      <c r="H43" s="82" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="59" t="inlineStr">
         <is>
           <t>Example 10</t>
         </is>
       </c>
-      <c r="B43" s="83" t="n"/>
-      <c r="C43" s="83" t="n"/>
-      <c r="D43" s="83" t="n"/>
-      <c r="E43" s="83" t="n"/>
-      <c r="F43" s="83" t="n"/>
-      <c r="G43" s="83" t="n"/>
-      <c r="H43" s="84" t="n"/>
+      <c r="B44" s="83" t="n"/>
+      <c r="C44" s="83" t="n"/>
+      <c r="D44" s="83" t="n"/>
+      <c r="E44" s="83" t="n"/>
+      <c r="F44" s="83" t="n"/>
+      <c r="G44" s="83" t="n"/>
+      <c r="H44" s="84" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="20">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="B15:H15"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B5:H5"/>
+    <mergeCell ref="B20:H20"/>
     <mergeCell ref="B4:H4"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B3:H3"/>
+    <mergeCell ref="A21:H21"/>
     <mergeCell ref="B18:H18"/>
+    <mergeCell ref="A33:H33"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="B11:H11"/>
-    <mergeCell ref="A32:H32"/>
     <mergeCell ref="B17:H17"/>
-    <mergeCell ref="A20:H20"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="B19:H19"/>
   </mergeCells>
   <dataValidations count="9">
-    <dataValidation sqref="F21:F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="F22:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"4°C,Dry Ice"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="G21:G30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="G22:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Discard,Return,Extended Storage"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="H21:H30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="H22:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1639,23 +1654,23 @@
       <formula1>"Mail,Drop Off,On Site (single cell only),Pick up (single cell only)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C34:C43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="C35:C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Water,EB"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B21:B30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="B22:B31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"RNA-Seq (mRNA),RNA-Seq (rRNA depletion),Single Cell (5'),Single Cell (3'),Single Cell (VDJ),Single Cell (5' + VDJ),Shotgun Meta,WGS,sequencing only"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="D21:D30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="D22:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Mouse,Human,Other (Please specify in Sample Note)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B34:B43" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="B35:B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Total RNA,cDNA library"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C21:C30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="C22:C31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Body Fluid,Cell,Tissue,Whole Blood,Nucleic Acid,Stool,Water,Soil,cDNA Library"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
split Analysis Purpose into required (purpose+comparison/baseline) vs optional (filtering/QC/stats) rows
Optional row: unspecified -> analyst applies default best-practice method.
Cross-references (row15/IMPORTANT/divider) updated for new row count.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
+++ b/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="38.44" customWidth="1" style="46" min="1" max="1"/>
@@ -1126,7 +1126,7 @@
       <c r="B15" s="73" t="inlineStr">
         <is>
           <t>Please read the following instructions, then delete all the default/sample text and input your own information and instructions.
-This section (rows 15-19) is your OVERALL submission information — what you want analyzed and how. Individual sample details go in the table below (see the "Per-Sample Details" section).</t>
+This section (rows 15-21) is your OVERALL submission information — what you want analyzed and how. Individual sample details go in the table below (see the "Per-Sample Details" section).</t>
         </is>
       </c>
       <c r="C15" s="64" t="n"/>
@@ -1180,21 +1180,20 @@
       <c r="A18" s="77" t="inlineStr">
         <is>
           <t>Analysis Purpose
-And Setting
-(list EACH
-requirement as its
-own numbered line)</t>
+and Comparisons
+(REQUIRED)</t>
         </is>
       </c>
       <c r="B18" s="78" t="inlineStr">
         <is>
-          <t xml:space="preserve">List EVERY requirement as its own numbered line below — e.g. analysis purpose, filtering/QC thresholds, groups to be compared, which is the control group (if applicable), statistical tests/significance thresholds, specific outputs needed. Do not combine multiple requirements into one line; add or delete numbered lines as needed.
+          <t xml:space="preserve">List your analysis purpose/objective(s), and for EACH comparison state which group is the baseline/reference (control). One item per numbered line — do not combine multiple items into one line.
+Example:
+1. Compare Group A (treated) vs Group B (control) — baseline/reference = Group B.
+2. Identify genes/features that differ significantly between Group A and Group B.
 1. 
 2. 
 3. 
-4. 
-5. 
-6. </t>
+4. </t>
         </is>
       </c>
       <c r="C18" s="64" t="n"/>
@@ -1204,30 +1203,59 @@
       <c r="G18" s="64" t="n"/>
       <c r="H18" s="65" t="n"/>
     </row>
-    <row r="19" ht="95" customHeight="1" s="47">
-      <c r="A19" s="79" t="inlineStr">
+    <row r="19" ht="130" customHeight="1" s="47">
+      <c r="A19" s="77" t="inlineStr">
+        <is>
+          <t>Filtering / QC /
+Statistical Thresholds
+(optional)</t>
+        </is>
+      </c>
+      <c r="B19" s="78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Optional — filtering/QC thresholds, statistical tests/significance thresholds, or other specific parameters (fill in only if you have a specific requirement).
+ℹ If you do NOT specify a value here, our analyst/statistician will apply the company's default / current statistical best-practice method for that analysis type, and will state the choice made in the final report.
+1. 
+2. 
+3. </t>
+        </is>
+      </c>
+      <c r="C19" s="64" t="n"/>
+      <c r="D19" s="64" t="n"/>
+      <c r="E19" s="64" t="n"/>
+      <c r="F19" s="64" t="n"/>
+      <c r="G19" s="64" t="n"/>
+      <c r="H19" s="65" t="n"/>
+    </row>
+    <row r="20" ht="110" customHeight="1" s="47">
+      <c r="A20" s="79" t="inlineStr">
         <is>
           <t>⚠ IMPORTANT
 (pricing basis)</t>
         </is>
       </c>
-      <c r="B19" s="80" t="inlineStr">
-        <is>
-          <t>⚠ IMPORTANT: This form — Sample Note +
-Analysis Type + Analysis Purpose and
-Setting above — is the SOLE basis for
+      <c r="B20" s="80" t="inlineStr">
+        <is>
+          <t>⚠ IMPORTANT: This form — Sample Note + Analysis Type +
+Analysis Purpose/Comparisons + Filtering/QC
+Thresholds above — is the SOLE basis for
 analysis scope and pricing. Requirements
 communicated only verbally or by email,
-and not written in the Analysis Purpose
-and Setting field above, will NOT be
+and not written in the fields above, will NOT be
 included in the analysis or the quote
 unless this form is updated and
 re-submitted.</t>
         </is>
       </c>
-    </row>
-    <row r="20" ht="165" customHeight="1" s="47">
-      <c r="A20" s="79" t="inlineStr">
+      <c r="C20" s="64" t="n"/>
+      <c r="D20" s="64" t="n"/>
+      <c r="E20" s="64" t="n"/>
+      <c r="F20" s="64" t="n"/>
+      <c r="G20" s="64" t="n"/>
+      <c r="H20" s="65" t="n"/>
+    </row>
+    <row r="21" ht="108" customHeight="1" s="47">
+      <c r="A21" s="79" t="inlineStr">
         <is>
           <t>Analysis requirements:
 Regular work for your selected category
@@ -1235,17 +1263,10 @@
 Custom requirements has Additional fee
 ($120/h).
 Our specialist will tell you which one is
-Custom item.
-ℹ If you do NOT specify a particular
-detail (e.g. a filtering threshold,
-statistical test, or significance cutoff),
-our analyst will apply the company's
-default / current statistical best-practice
-method for that analysis type, and will
-state the choice made in the final report.</t>
-        </is>
-      </c>
-      <c r="B20" s="80" t="inlineStr">
+Custom item.</t>
+        </is>
+      </c>
+      <c r="B21" s="80" t="inlineStr">
         <is>
           <t>For example, the following item is regular items for wgs : 
 * Call germline short variants (SNV/indel) genome-wide and annotate them for population rarity (gnomAD) and clinical significance (ClinVar).
@@ -1256,20 +1277,6 @@
 * Perform HLA genotyping (class I and class II) from the WGS data.</t>
         </is>
       </c>
-      <c r="C20" s="64" t="n"/>
-      <c r="D20" s="64" t="n"/>
-      <c r="E20" s="64" t="n"/>
-      <c r="F20" s="64" t="n"/>
-      <c r="G20" s="64" t="n"/>
-      <c r="H20" s="65" t="n"/>
-    </row>
-    <row r="21" ht="32" customHeight="1" s="47">
-      <c r="A21" s="109" t="inlineStr">
-        <is>
-          <t>▼ PER-SAMPLE DETAILS (below) — one row per individual physical sample.  The section above (rows 15-19) covers your overall submission: sample description, analysis type, and requirements.</t>
-        </is>
-      </c>
-      <c r="B21" s="64" t="n"/>
       <c r="C21" s="64" t="n"/>
       <c r="D21" s="64" t="n"/>
       <c r="E21" s="64" t="n"/>
@@ -1277,24 +1284,24 @@
       <c r="G21" s="64" t="n"/>
       <c r="H21" s="65" t="n"/>
     </row>
-    <row r="22" ht="15" customHeight="1" s="47">
-      <c r="A22" s="55" t="inlineStr">
-        <is>
-          <t>Example 1</t>
-        </is>
-      </c>
-      <c r="B22" s="81" t="n"/>
-      <c r="C22" s="81" t="n"/>
-      <c r="D22" s="81" t="n"/>
-      <c r="E22" s="81" t="n"/>
-      <c r="F22" s="81" t="n"/>
-      <c r="G22" s="81" t="n"/>
-      <c r="H22" s="82" t="n"/>
+    <row r="22" ht="32" customHeight="1" s="47">
+      <c r="A22" s="109" t="inlineStr">
+        <is>
+          <t>▼ PER-SAMPLE DETAILS (below) — one row per individual physical sample.  The section above (rows 15-19) covers your overall submission: sample description, analysis type, and requirements.</t>
+        </is>
+      </c>
+      <c r="B22" s="64" t="n"/>
+      <c r="C22" s="64" t="n"/>
+      <c r="D22" s="64" t="n"/>
+      <c r="E22" s="64" t="n"/>
+      <c r="F22" s="64" t="n"/>
+      <c r="G22" s="64" t="n"/>
+      <c r="H22" s="65" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="47">
       <c r="A23" s="55" t="inlineStr">
         <is>
-          <t>Example 2</t>
+          <t>Example 1</t>
         </is>
       </c>
       <c r="B23" s="81" t="n"/>
@@ -1308,7 +1315,7 @@
     <row r="24" ht="15" customHeight="1" s="47">
       <c r="A24" s="55" t="inlineStr">
         <is>
-          <t>Example 3</t>
+          <t>Example 2</t>
         </is>
       </c>
       <c r="B24" s="81" t="n"/>
@@ -1322,7 +1329,7 @@
     <row r="25" ht="15" customHeight="1" s="47">
       <c r="A25" s="55" t="inlineStr">
         <is>
-          <t>Example 4</t>
+          <t>Example 3</t>
         </is>
       </c>
       <c r="B25" s="81" t="n"/>
@@ -1336,7 +1343,7 @@
     <row r="26" ht="15" customHeight="1" s="47">
       <c r="A26" s="55" t="inlineStr">
         <is>
-          <t>Example 5</t>
+          <t>Example 4</t>
         </is>
       </c>
       <c r="B26" s="81" t="n"/>
@@ -1350,7 +1357,7 @@
     <row r="27" ht="15" customHeight="1" s="47">
       <c r="A27" s="55" t="inlineStr">
         <is>
-          <t>Example 6</t>
+          <t>Example 5</t>
         </is>
       </c>
       <c r="B27" s="81" t="n"/>
@@ -1364,7 +1371,7 @@
     <row r="28" ht="15" customHeight="1" s="47">
       <c r="A28" s="55" t="inlineStr">
         <is>
-          <t>Example 7</t>
+          <t>Example 6</t>
         </is>
       </c>
       <c r="B28" s="81" t="n"/>
@@ -1378,7 +1385,7 @@
     <row r="29" ht="15" customHeight="1" s="47">
       <c r="A29" s="55" t="inlineStr">
         <is>
-          <t>Example 8</t>
+          <t>Example 7</t>
         </is>
       </c>
       <c r="B29" s="81" t="n"/>
@@ -1392,7 +1399,7 @@
     <row r="30" ht="15" customHeight="1" s="47">
       <c r="A30" s="55" t="inlineStr">
         <is>
-          <t>Example 9</t>
+          <t>Example 8</t>
         </is>
       </c>
       <c r="B30" s="81" t="n"/>
@@ -1404,94 +1411,94 @@
       <c r="H30" s="82" t="n"/>
     </row>
     <row r="31" ht="15" customHeight="1" s="47">
-      <c r="A31" s="59" t="inlineStr">
+      <c r="A31" s="55" t="inlineStr">
+        <is>
+          <t>Example 9</t>
+        </is>
+      </c>
+      <c r="B31" s="81" t="n"/>
+      <c r="C31" s="81" t="n"/>
+      <c r="D31" s="81" t="n"/>
+      <c r="E31" s="81" t="n"/>
+      <c r="F31" s="81" t="n"/>
+      <c r="G31" s="81" t="n"/>
+      <c r="H31" s="82" t="n"/>
+    </row>
+    <row r="32" ht="15" customHeight="1" s="47">
+      <c r="A32" s="59" t="inlineStr">
         <is>
           <t>Example 10</t>
         </is>
       </c>
-      <c r="B31" s="83" t="n"/>
-      <c r="C31" s="83" t="n"/>
-      <c r="D31" s="83" t="n"/>
-      <c r="E31" s="83" t="n"/>
-      <c r="F31" s="83" t="n"/>
-      <c r="G31" s="83" t="n"/>
-      <c r="H31" s="84" t="n"/>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="47"/>
-    <row r="33" ht="14.25" customHeight="1" s="47">
-      <c r="A33" s="63" t="inlineStr">
+      <c r="B32" s="83" t="n"/>
+      <c r="C32" s="83" t="n"/>
+      <c r="D32" s="83" t="n"/>
+      <c r="E32" s="83" t="n"/>
+      <c r="F32" s="83" t="n"/>
+      <c r="G32" s="83" t="n"/>
+      <c r="H32" s="84" t="n"/>
+    </row>
+    <row r="33" ht="15" customHeight="1" s="47"/>
+    <row r="34" ht="14.25" customHeight="1" s="47">
+      <c r="A34" s="63" t="inlineStr">
         <is>
           <t>Nucleic Acids Additional Information</t>
         </is>
       </c>
-      <c r="B33" s="64" t="n"/>
-      <c r="C33" s="64" t="n"/>
-      <c r="D33" s="64" t="n"/>
-      <c r="E33" s="64" t="n"/>
-      <c r="F33" s="64" t="n"/>
-      <c r="G33" s="64" t="n"/>
-      <c r="H33" s="65" t="n"/>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="47">
-      <c r="A34" s="66" t="inlineStr">
+      <c r="B34" s="64" t="n"/>
+      <c r="C34" s="64" t="n"/>
+      <c r="D34" s="64" t="n"/>
+      <c r="E34" s="64" t="n"/>
+      <c r="F34" s="64" t="n"/>
+      <c r="G34" s="64" t="n"/>
+      <c r="H34" s="65" t="n"/>
+    </row>
+    <row r="35" ht="15" customHeight="1" s="47">
+      <c r="A35" s="66" t="inlineStr">
         <is>
           <t>Sample Name</t>
         </is>
       </c>
-      <c r="B34" s="85" t="inlineStr">
+      <c r="B35" s="85" t="inlineStr">
         <is>
           <t>Nucleic Acid Type</t>
         </is>
       </c>
-      <c r="C34" s="85" t="inlineStr">
+      <c r="C35" s="85" t="inlineStr">
         <is>
           <t>Storage Reagent</t>
         </is>
       </c>
-      <c r="D34" s="85" t="inlineStr">
+      <c r="D35" s="85" t="inlineStr">
         <is>
           <t>Concentration (ng/µL)</t>
         </is>
       </c>
-      <c r="E34" s="85" t="inlineStr">
+      <c r="E35" s="85" t="inlineStr">
         <is>
           <t>Volume (µL)</t>
         </is>
       </c>
-      <c r="F34" s="85" t="inlineStr">
+      <c r="F35" s="85" t="inlineStr">
         <is>
           <t>Size (bp, if applicable)</t>
         </is>
       </c>
-      <c r="G34" s="85" t="inlineStr">
+      <c r="G35" s="85" t="inlineStr">
         <is>
           <t>i7 Index (if any)</t>
         </is>
       </c>
-      <c r="H34" s="86" t="inlineStr">
+      <c r="H35" s="86" t="inlineStr">
         <is>
           <t>i5 Index (NovaSeq 1.0/Forward)</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="47">
-      <c r="A35" s="55" t="inlineStr">
+    <row r="36" ht="15" customHeight="1" s="47">
+      <c r="A36" s="55" t="inlineStr">
         <is>
           <t>Example 1</t>
-        </is>
-      </c>
-      <c r="B35" s="81" t="n"/>
-      <c r="C35" s="81" t="n"/>
-      <c r="D35" s="81" t="n"/>
-      <c r="E35" s="81" t="n"/>
-      <c r="F35" s="81" t="n"/>
-      <c r="G35" s="81" t="n"/>
-      <c r="H35" s="82" t="n"/>
-    </row>
-    <row r="36" ht="14.25" customHeight="1" s="47">
-      <c r="A36" s="55" t="inlineStr">
-        <is>
-          <t>Example 2</t>
         </is>
       </c>
       <c r="B36" s="81" t="n"/>
@@ -1505,7 +1512,7 @@
     <row r="37" ht="14.25" customHeight="1" s="47">
       <c r="A37" s="55" t="inlineStr">
         <is>
-          <t>Example 3</t>
+          <t>Example 2</t>
         </is>
       </c>
       <c r="B37" s="81" t="n"/>
@@ -1519,7 +1526,7 @@
     <row r="38" ht="14.25" customHeight="1" s="47">
       <c r="A38" s="55" t="inlineStr">
         <is>
-          <t>Example 4</t>
+          <t>Example 3</t>
         </is>
       </c>
       <c r="B38" s="81" t="n"/>
@@ -1533,7 +1540,7 @@
     <row r="39" ht="14.25" customHeight="1" s="47">
       <c r="A39" s="55" t="inlineStr">
         <is>
-          <t>Example 5</t>
+          <t>Example 4</t>
         </is>
       </c>
       <c r="B39" s="81" t="n"/>
@@ -1547,7 +1554,7 @@
     <row r="40" ht="14.25" customHeight="1" s="47">
       <c r="A40" s="55" t="inlineStr">
         <is>
-          <t>Example 6</t>
+          <t>Example 5</t>
         </is>
       </c>
       <c r="B40" s="81" t="n"/>
@@ -1561,7 +1568,7 @@
     <row r="41" ht="14.25" customHeight="1" s="47">
       <c r="A41" s="55" t="inlineStr">
         <is>
-          <t>Example 7</t>
+          <t>Example 6</t>
         </is>
       </c>
       <c r="B41" s="81" t="n"/>
@@ -1575,7 +1582,7 @@
     <row r="42" ht="14.25" customHeight="1" s="47">
       <c r="A42" s="55" t="inlineStr">
         <is>
-          <t>Example 8</t>
+          <t>Example 7</t>
         </is>
       </c>
       <c r="B42" s="81" t="n"/>
@@ -1586,10 +1593,10 @@
       <c r="G42" s="81" t="n"/>
       <c r="H42" s="82" t="n"/>
     </row>
-    <row r="43" ht="15" customHeight="1" s="47">
+    <row r="43" ht="14.25" customHeight="1" s="47">
       <c r="A43" s="55" t="inlineStr">
         <is>
-          <t>Example 9</t>
+          <t>Example 8</t>
         </is>
       </c>
       <c r="B43" s="81" t="n"/>
@@ -1600,22 +1607,36 @@
       <c r="G43" s="81" t="n"/>
       <c r="H43" s="82" t="n"/>
     </row>
-    <row r="44">
-      <c r="A44" s="59" t="inlineStr">
+    <row r="44" ht="15" customHeight="1" s="47">
+      <c r="A44" s="55" t="inlineStr">
+        <is>
+          <t>Example 9</t>
+        </is>
+      </c>
+      <c r="B44" s="81" t="n"/>
+      <c r="C44" s="81" t="n"/>
+      <c r="D44" s="81" t="n"/>
+      <c r="E44" s="81" t="n"/>
+      <c r="F44" s="81" t="n"/>
+      <c r="G44" s="81" t="n"/>
+      <c r="H44" s="82" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="59" t="inlineStr">
         <is>
           <t>Example 10</t>
         </is>
       </c>
-      <c r="B44" s="83" t="n"/>
-      <c r="C44" s="83" t="n"/>
-      <c r="D44" s="83" t="n"/>
-      <c r="E44" s="83" t="n"/>
-      <c r="F44" s="83" t="n"/>
-      <c r="G44" s="83" t="n"/>
-      <c r="H44" s="84" t="n"/>
+      <c r="B45" s="83" t="n"/>
+      <c r="C45" s="83" t="n"/>
+      <c r="D45" s="83" t="n"/>
+      <c r="E45" s="83" t="n"/>
+      <c r="F45" s="83" t="n"/>
+      <c r="G45" s="83" t="n"/>
+      <c r="H45" s="84" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="21">
     <mergeCell ref="A9:H9"/>
     <mergeCell ref="B6:H6"/>
     <mergeCell ref="B15:H15"/>
@@ -1626,27 +1647,28 @@
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B3:H3"/>
-    <mergeCell ref="A21:H21"/>
     <mergeCell ref="B18:H18"/>
-    <mergeCell ref="A33:H33"/>
+    <mergeCell ref="B21:H21"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="B11:H11"/>
+    <mergeCell ref="A22:H22"/>
     <mergeCell ref="B17:H17"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="B10:H10"/>
     <mergeCell ref="B19:H19"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <dataValidations count="9">
-    <dataValidation sqref="F22:F31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="F23:F32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"4°C,Dry Ice"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="G22:G31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="G23:G32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Discard,Return,Extended Storage"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="H22:H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="H23:H32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1654,23 +1676,23 @@
       <formula1>"Mail,Drop Off,On Site (single cell only),Pick up (single cell only)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C35:C44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="C36:C45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Water,EB"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B22:B31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="B23:B32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"RNA-Seq (mRNA),RNA-Seq (rRNA depletion),Single Cell (5'),Single Cell (3'),Single Cell (VDJ),Single Cell (5' + VDJ),Shotgun Meta,WGS,sequencing only"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="D22:D31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="D23:D32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Mouse,Human,Other (Please specify in Sample Note)"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B35:B44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="B36:B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Total RNA,cDNA library"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="C22:C31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
+    <dataValidation sqref="C23:C32" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" operator="between">
       <formula1>"Body Fluid,Cell,Tissue,Whole Blood,Nucleic Acid,Stool,Water,Soil,cDNA Library"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
unify row 15-21 alignment/heights, restore+expand service list, generalize example
Analysis Type: merge original list with per-sample dropdown categories +
common services (epigenomics, microbiome, long-read, etc).
Row19 text: professional tone, drop info-emoji for consistency.
Row21 example: WGS-specific -> analysis-type-agnostic.
Row heights: computed from text length instead of guessed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
+++ b/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
@@ -374,7 +374,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="110">
+  <cellXfs count="114">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -666,6 +666,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1117,13 +1129,13 @@
       <c r="G14" s="64" t="n"/>
       <c r="H14" s="65" t="n"/>
     </row>
-    <row r="15" ht="16.15" customHeight="1" s="47">
-      <c r="A15" s="72" t="inlineStr">
+    <row r="15" ht="87.5" customHeight="1" s="47">
+      <c r="A15" s="77" t="inlineStr">
         <is>
           <t>Sample Information and instruction</t>
         </is>
       </c>
-      <c r="B15" s="73" t="inlineStr">
+      <c r="B15" s="110" t="inlineStr">
         <is>
           <t>Please read the following instructions, then delete all the default/sample text and input your own information and instructions.
 This section (rows 15-21) is your OVERALL submission information — what you want analyzed and how. Individual sample details go in the table below (see the "Per-Sample Details" section).</t>
@@ -1136,13 +1148,13 @@
       <c r="G15" s="64" t="n"/>
       <c r="H15" s="74" t="n"/>
     </row>
-    <row r="16" ht="30.85" customHeight="1" s="47">
-      <c r="A16" s="72" t="inlineStr">
+    <row r="16" ht="87.5" customHeight="1" s="47">
+      <c r="A16" s="77" t="inlineStr">
         <is>
           <t>Sample Note:</t>
         </is>
       </c>
-      <c r="B16" s="75" t="inlineStr">
+      <c r="B16" s="111" t="inlineStr">
         <is>
           <t>Please specify the source of sample in general, as detail as possible, such as 
 Cell line, organ, tissue, iPSCs, humanized mice, human cells expressed in mice, tumor/normal, stool, blood, brain etc.
@@ -1156,16 +1168,21 @@
       <c r="G16" s="64" t="n"/>
       <c r="H16" s="74" t="n"/>
     </row>
-    <row r="17" ht="26.05" customHeight="1" s="47">
-      <c r="A17" s="72" t="inlineStr">
+    <row r="17" ht="289" customHeight="1" s="47">
+      <c r="A17" s="77" t="inlineStr">
         <is>
           <t>Analysis Type :</t>
         </is>
       </c>
-      <c r="B17" s="76" t="inlineStr">
-        <is>
-          <t>The analysis type (input only ONE type of analysis), such as 
-RNAseq,  Single-Cell-Analysis, spatial Transcriptomics, whole-genome-sequence, proteomics, mapping based or assembly-based shotgun metagenomics
+      <c r="B17" s="112" t="inlineStr">
+        <is>
+          <t>The analysis type — input ONE type per form (see note below for multi-part submissions). Our common service categories include:
+• Transcriptomics: Bulk RNA-Seq (mRNA / total RNA / rRNA-depletion), Single-Cell RNA-Seq (3', 5', VDJ), Spatial Transcriptomics, Small RNA-Seq
+• Genome Sequencing: Whole-Genome Sequencing (WGS), Whole-Exome Sequencing (WES), de novo Genome Assembly, Long-Read Sequencing (PacBio/Nanopore)
+• Epigenomics: ATAC-Seq, ChIP-Seq, Whole-Genome Bisulfite Sequencing (WGBS) / DNA Methylation
+• Microbiome and Metagenomics: 16S/18S/ITS Amplicon Sequencing, Shotgun Metagenomics (mapping-based or assembly-based / MAG)
+• Other Services: Proteomics, HLA Genotyping, Sanger Sequencing, Plasmid/Construct Verification, Sequencing Only (no bioinformatics analysis)
+Don't see your service listed here? Describe it in your own words — we support most standard and custom sequencing and analysis workflows.
 ⚠ If this submission includes two different analysis types or two distinct parts (e.g. RNAseq AND WGS, or two separate studies), please fill out and submit TWO separate copies of this form, one per analysis type / part.</t>
         </is>
       </c>
@@ -1176,7 +1193,7 @@
       <c r="G17" s="64" t="n"/>
       <c r="H17" s="65" t="n"/>
     </row>
-    <row r="18" ht="165" customHeight="1" s="47">
+    <row r="18" ht="180.5" customHeight="1" s="47">
       <c r="A18" s="77" t="inlineStr">
         <is>
           <t>Analysis Purpose
@@ -1184,7 +1201,7 @@
 (REQUIRED)</t>
         </is>
       </c>
-      <c r="B18" s="78" t="inlineStr">
+      <c r="B18" s="112" t="inlineStr">
         <is>
           <t xml:space="preserve">List your analysis purpose/objective(s), and for EACH comparison state which group is the baseline/reference (control). One item per numbered line — do not combine multiple items into one line.
 Example:
@@ -1203,7 +1220,7 @@
       <c r="G18" s="64" t="n"/>
       <c r="H18" s="65" t="n"/>
     </row>
-    <row r="19" ht="130" customHeight="1" s="47">
+    <row r="19" ht="149.5" customHeight="1" s="47">
       <c r="A19" s="77" t="inlineStr">
         <is>
           <t>Filtering / QC /
@@ -1211,10 +1228,10 @@
 (optional)</t>
         </is>
       </c>
-      <c r="B19" s="78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Optional — filtering/QC thresholds, statistical tests/significance thresholds, or other specific parameters (fill in only if you have a specific requirement).
-ℹ If you do NOT specify a value here, our analyst/statistician will apply the company's default / current statistical best-practice method for that analysis type, and will state the choice made in the final report.
+      <c r="B19" s="112" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Filtering, quality-control thresholds, statistical test selection, and significance cutoffs for this analysis — optional; provide only if you have a specific requirement.
+If a value is not specified, our analyst will apply the current standard / default methodology for the selected analysis type and document the choice made in the final report.
 1. 
 2. 
 3. </t>
@@ -1227,14 +1244,14 @@
       <c r="G19" s="64" t="n"/>
       <c r="H19" s="65" t="n"/>
     </row>
-    <row r="20" ht="110" customHeight="1" s="47">
-      <c r="A20" s="79" t="inlineStr">
+    <row r="20" ht="149.5" customHeight="1" s="47">
+      <c r="A20" s="77" t="inlineStr">
         <is>
           <t>⚠ IMPORTANT
 (pricing basis)</t>
         </is>
       </c>
-      <c r="B20" s="80" t="inlineStr">
+      <c r="B20" s="113" t="inlineStr">
         <is>
           <t>⚠ IMPORTANT: This form — Sample Note + Analysis Type +
 Analysis Purpose/Comparisons + Filtering/QC
@@ -1254,8 +1271,8 @@
       <c r="G20" s="64" t="n"/>
       <c r="H20" s="65" t="n"/>
     </row>
-    <row r="21" ht="108" customHeight="1" s="47">
-      <c r="A21" s="79" t="inlineStr">
+    <row r="21" ht="180.5" customHeight="1" s="47">
+      <c r="A21" s="77" t="inlineStr">
         <is>
           <t>Analysis requirements:
 Regular work for your selected category
@@ -1266,15 +1283,11 @@
 Custom item.</t>
         </is>
       </c>
-      <c r="B21" s="80" t="inlineStr">
-        <is>
-          <t>For example, the following item is regular items for wgs : 
-* Call germline short variants (SNV/indel) genome-wide and annotate them for population rarity (gnomAD) and clinical significance (ClinVar).
-* Prioritise a shortlist of rare and potentially functional / clinically relevant variants.
-* Call structural variants (SV) and copy-number variants (CNV).
-* Infer, from the data alone, whether the material is more consistent with primary/germline tissue or a passaged cell line (the client did not specify tissue of origin)
-The flowing item is costom item:  
-* Perform HLA genotyping (class I and class II) from the WGS data.</t>
+      <c r="B21" s="113" t="inlineStr">
+        <is>
+          <t>For example, across most analysis types: standard outputs covered by our default pipeline for your selected Analysis Type — e.g. QC reports, standard alignment/quantification, comparative analysis using our default statistical methods (see Filtering/QC/Statistical Thresholds above), and a written summary report — are Regular (no extra fee).
+Requests beyond that default pipeline — additional analyses not covered by the standard workflow, custom scripts or pipelines, extra comparisons beyond what you specified, or specialized add-on modules (e.g. HLA genotyping on WGS data, custom visualizations, extended consulting) — are Custom ($120/h).
+Our specialist will confirm, for your specific Analysis Purpose and Comparisons above, which items fall into each category before work begins.</t>
         </is>
       </c>
       <c r="C21" s="64" t="n"/>

</xml_diff>

<commit_message>
fix IMPORTANT row: reflow text (was hard-wrapped for narrow column), recompute height
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
+++ b/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
@@ -1244,7 +1244,7 @@
       <c r="G19" s="64" t="n"/>
       <c r="H19" s="65" t="n"/>
     </row>
-    <row r="20" ht="149.5" customHeight="1" s="47">
+    <row r="20" ht="56.5" customHeight="1" s="47">
       <c r="A20" s="77" t="inlineStr">
         <is>
           <t>⚠ IMPORTANT
@@ -1253,15 +1253,7 @@
       </c>
       <c r="B20" s="113" t="inlineStr">
         <is>
-          <t>⚠ IMPORTANT: This form — Sample Note + Analysis Type +
-Analysis Purpose/Comparisons + Filtering/QC
-Thresholds above — is the SOLE basis for
-analysis scope and pricing. Requirements
-communicated only verbally or by email,
-and not written in the fields above, will NOT be
-included in the analysis or the quote
-unless this form is updated and
-re-submitted.</t>
+          <t>This form — Sample Note, Analysis Type, Analysis Purpose and Comparisons, and Filtering/QC/Statistical Thresholds above — is the SOLE basis for analysis scope and pricing. Requirements communicated only verbally or by email, and not written in the fields above, will NOT be included in the analysis or the quote unless this form is updated and re-submitted.</t>
         </is>
       </c>
       <c r="C20" s="64" t="n"/>

</xml_diff>

<commit_message>
unify page-1 font: Calibri 11 everywhere, bold labels/regular content
Drop red on 6 labels (was diluting the signal) and oversized blue B15;
keep red bold ONLY on the IMPORTANT pricing row as the one highlight.
Fix empty font-name defect on B20/B21 (inherited from original template).
Add paragraph spacing to B21 (Analysis requirements example).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
+++ b/facilities/AI_and_Agent/Company/Sample_Registration_Form_ZG.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -93,6 +93,21 @@
       <sz val="11"/>
     </font>
     <font/>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFC9211E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -374,7 +389,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -678,6 +693,42 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -960,7 +1011,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1" s="47">
-      <c r="A1" s="48" t="inlineStr">
+      <c r="A1" s="114" t="inlineStr">
         <is>
           <t>Customer Information</t>
         </is>
@@ -974,7 +1025,7 @@
       <c r="H1" s="50" t="n"/>
     </row>
     <row r="2" ht="14.25" customHeight="1" s="47">
-      <c r="A2" s="51" t="inlineStr">
+      <c r="A2" s="115" t="inlineStr">
         <is>
           <t>Quote Number</t>
         </is>
@@ -988,7 +1039,7 @@
       <c r="H2" s="54" t="n"/>
     </row>
     <row r="3" ht="14.25" customHeight="1" s="47">
-      <c r="A3" s="55" t="inlineStr">
+      <c r="A3" s="116" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
@@ -1002,7 +1053,7 @@
       <c r="H3" s="58" t="n"/>
     </row>
     <row r="4" ht="14.25" customHeight="1" s="47">
-      <c r="A4" s="55" t="inlineStr">
+      <c r="A4" s="116" t="inlineStr">
         <is>
           <t>Organization</t>
         </is>
@@ -1016,7 +1067,7 @@
       <c r="H4" s="58" t="n"/>
     </row>
     <row r="5" ht="14.25" customHeight="1" s="47">
-      <c r="A5" s="55" t="inlineStr">
+      <c r="A5" s="116" t="inlineStr">
         <is>
           <t>Phone</t>
         </is>
@@ -1030,7 +1081,7 @@
       <c r="H5" s="58" t="n"/>
     </row>
     <row r="6" ht="14.25" customHeight="1" s="47">
-      <c r="A6" s="55" t="inlineStr">
+      <c r="A6" s="116" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
@@ -1044,7 +1095,7 @@
       <c r="H6" s="58" t="n"/>
     </row>
     <row r="7" ht="15" customHeight="1" s="47">
-      <c r="A7" s="59" t="inlineStr">
+      <c r="A7" s="117" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
@@ -1059,7 +1110,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" s="47"/>
     <row r="9" ht="15" customHeight="1" s="47">
-      <c r="A9" s="63" t="inlineStr">
+      <c r="A9" s="118" t="inlineStr">
         <is>
           <t>Delivery Information</t>
         </is>
@@ -1073,7 +1124,7 @@
       <c r="H9" s="65" t="n"/>
     </row>
     <row r="10" ht="14.25" customHeight="1" s="47">
-      <c r="A10" s="66" t="inlineStr">
+      <c r="A10" s="119" t="inlineStr">
         <is>
           <t>Delivery Method</t>
         </is>
@@ -1087,7 +1138,7 @@
       <c r="H10" s="69" t="n"/>
     </row>
     <row r="11" ht="15" customHeight="1" s="47">
-      <c r="A11" s="59" t="inlineStr">
+      <c r="A11" s="117" t="inlineStr">
         <is>
           <t>Delivery Note</t>
         </is>
@@ -1102,7 +1153,7 @@
     </row>
     <row r="12" ht="14.25" customHeight="1" s="47"/>
     <row r="13" ht="15" customHeight="1" s="47">
-      <c r="A13" s="63" t="inlineStr">
+      <c r="A13" s="118" t="inlineStr">
         <is>
           <t>Project:</t>
         </is>
@@ -1116,7 +1167,7 @@
       <c r="H13" s="65" t="n"/>
     </row>
     <row r="14" ht="15" customHeight="1" s="47">
-      <c r="A14" s="71" t="inlineStr">
+      <c r="A14" s="118" t="inlineStr">
         <is>
           <t>Expected Delivery Date:</t>
         </is>
@@ -1130,12 +1181,12 @@
       <c r="H14" s="65" t="n"/>
     </row>
     <row r="15" ht="87.5" customHeight="1" s="47">
-      <c r="A15" s="77" t="inlineStr">
+      <c r="A15" s="120" t="inlineStr">
         <is>
           <t>Sample Information and instruction</t>
         </is>
       </c>
-      <c r="B15" s="110" t="inlineStr">
+      <c r="B15" s="121" t="inlineStr">
         <is>
           <t>Please read the following instructions, then delete all the default/sample text and input your own information and instructions.
 This section (rows 15-21) is your OVERALL submission information — what you want analyzed and how. Individual sample details go in the table below (see the "Per-Sample Details" section).</t>
@@ -1149,12 +1200,12 @@
       <c r="H15" s="74" t="n"/>
     </row>
     <row r="16" ht="87.5" customHeight="1" s="47">
-      <c r="A16" s="77" t="inlineStr">
+      <c r="A16" s="120" t="inlineStr">
         <is>
           <t>Sample Note:</t>
         </is>
       </c>
-      <c r="B16" s="111" t="inlineStr">
+      <c r="B16" s="122" t="inlineStr">
         <is>
           <t>Please specify the source of sample in general, as detail as possible, such as 
 Cell line, organ, tissue, iPSCs, humanized mice, human cells expressed in mice, tumor/normal, stool, blood, brain etc.
@@ -1169,12 +1220,12 @@
       <c r="H16" s="74" t="n"/>
     </row>
     <row r="17" ht="289" customHeight="1" s="47">
-      <c r="A17" s="77" t="inlineStr">
+      <c r="A17" s="120" t="inlineStr">
         <is>
           <t>Analysis Type :</t>
         </is>
       </c>
-      <c r="B17" s="112" t="inlineStr">
+      <c r="B17" s="123" t="inlineStr">
         <is>
           <t>The analysis type — input ONE type per form (see note below for multi-part submissions). Our common service categories include:
 • Transcriptomics: Bulk RNA-Seq (mRNA / total RNA / rRNA-depletion), Single-Cell RNA-Seq (3', 5', VDJ), Spatial Transcriptomics, Small RNA-Seq
@@ -1194,14 +1245,14 @@
       <c r="H17" s="65" t="n"/>
     </row>
     <row r="18" ht="180.5" customHeight="1" s="47">
-      <c r="A18" s="77" t="inlineStr">
+      <c r="A18" s="120" t="inlineStr">
         <is>
           <t>Analysis Purpose
 and Comparisons
 (REQUIRED)</t>
         </is>
       </c>
-      <c r="B18" s="112" t="inlineStr">
+      <c r="B18" s="123" t="inlineStr">
         <is>
           <t xml:space="preserve">List your analysis purpose/objective(s), and for EACH comparison state which group is the baseline/reference (control). One item per numbered line — do not combine multiple items into one line.
 Example:
@@ -1221,14 +1272,14 @@
       <c r="H18" s="65" t="n"/>
     </row>
     <row r="19" ht="149.5" customHeight="1" s="47">
-      <c r="A19" s="77" t="inlineStr">
+      <c r="A19" s="120" t="inlineStr">
         <is>
           <t>Filtering / QC /
 Statistical Thresholds
 (optional)</t>
         </is>
       </c>
-      <c r="B19" s="112" t="inlineStr">
+      <c r="B19" s="123" t="inlineStr">
         <is>
           <t xml:space="preserve">Filtering, quality-control thresholds, statistical test selection, and significance cutoffs for this analysis — optional; provide only if you have a specific requirement.
 If a value is not specified, our analyst will apply the current standard / default methodology for the selected analysis type and document the choice made in the final report.
@@ -1245,13 +1296,13 @@
       <c r="H19" s="65" t="n"/>
     </row>
     <row r="20" ht="56.5" customHeight="1" s="47">
-      <c r="A20" s="77" t="inlineStr">
+      <c r="A20" s="124" t="inlineStr">
         <is>
           <t>⚠ IMPORTANT
 (pricing basis)</t>
         </is>
       </c>
-      <c r="B20" s="113" t="inlineStr">
+      <c r="B20" s="123" t="inlineStr">
         <is>
           <t>This form — Sample Note, Analysis Type, Analysis Purpose and Comparisons, and Filtering/QC/Statistical Thresholds above — is the SOLE basis for analysis scope and pricing. Requirements communicated only verbally or by email, and not written in the fields above, will NOT be included in the analysis or the quote unless this form is updated and re-submitted.</t>
         </is>
@@ -1264,7 +1315,7 @@
       <c r="H20" s="65" t="n"/>
     </row>
     <row r="21" ht="180.5" customHeight="1" s="47">
-      <c r="A21" s="77" t="inlineStr">
+      <c r="A21" s="120" t="inlineStr">
         <is>
           <t>Analysis requirements:
 Regular work for your selected category
@@ -1275,7 +1326,7 @@
 Custom item.</t>
         </is>
       </c>
-      <c r="B21" s="113" t="inlineStr">
+      <c r="B21" s="123" t="inlineStr">
         <is>
           <t>For example, across most analysis types: standard outputs covered by our default pipeline for your selected Analysis Type — e.g. QC reports, standard alignment/quantification, comparative analysis using our default statistical methods (see Filtering/QC/Statistical Thresholds above), and a written summary report — are Regular (no extra fee).
 Requests beyond that default pipeline — additional analyses not covered by the standard workflow, custom scripts or pipelines, extra comparisons beyond what you specified, or specialized add-on modules (e.g. HLA genotyping on WGS data, custom visualizations, extended consulting) — are Custom ($120/h).
@@ -1290,7 +1341,7 @@
       <c r="H21" s="65" t="n"/>
     </row>
     <row r="22" ht="32" customHeight="1" s="47">
-      <c r="A22" s="109" t="inlineStr">
+      <c r="A22" s="125" t="inlineStr">
         <is>
           <t>▼ PER-SAMPLE DETAILS (below) — one row per individual physical sample.  The section above (rows 15-19) covers your overall submission: sample description, analysis type, and requirements.</t>
         </is>

</xml_diff>